<commit_message>
double pair to size optimize wvshape
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF349C1-6EBF-48D5-930C-18E73546A464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B053404-0A65-4AF5-B723-9FA5E9991218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8640" yWindow="225" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -97,6 +97,12 @@
   </si>
   <si>
     <t>clamp noinline</t>
+  </si>
+  <si>
+    <t>no unique_ptr</t>
+  </si>
+  <si>
+    <t>weird doublepair refact</t>
   </si>
 </sst>
 </file>
@@ -467,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -613,7 +619,7 @@
         <v>37392</v>
       </c>
       <c r="D7" s="2">
-        <f t="shared" ref="D7:D19" si="3">C6-C7</f>
+        <f t="shared" ref="D7:D21" si="3">C6-C7</f>
         <v>-16</v>
       </c>
       <c r="E7">
@@ -964,6 +970,46 @@
         <v>23</v>
       </c>
     </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>34188</v>
+      </c>
+      <c r="D20" s="2">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="E20">
+        <f t="shared" ref="E20" si="29">$C$4-C20</f>
+        <v>4212</v>
+      </c>
+      <c r="F20">
+        <f t="shared" ref="F20" si="30">$O$2-C20</f>
+        <v>-1420</v>
+      </c>
+      <c r="G20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>34132</v>
+      </c>
+      <c r="D21" s="2">
+        <f t="shared" si="3"/>
+        <v>56</v>
+      </c>
+      <c r="E21">
+        <f t="shared" ref="E21" si="31">$C$4-C21</f>
+        <v>4268</v>
+      </c>
+      <c r="F21">
+        <f t="shared" ref="F21" si="32">$O$2-C21</f>
+        <v>-1364</v>
+      </c>
+      <c r="G21" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
removing enum class width
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B053404-0A65-4AF5-B723-9FA5E9991218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D5952B-A0CC-4CA8-9153-138B72DF6859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8640" yWindow="225" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -103,6 +103,12 @@
   </si>
   <si>
     <t>weird doublepair refact</t>
+  </si>
+  <si>
+    <t>de-inlining vwshape</t>
+  </si>
+  <si>
+    <t>removing uint8_t enum class</t>
   </si>
 </sst>
 </file>
@@ -473,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -532,7 +538,7 @@
         <v>5632</v>
       </c>
       <c r="B4" s="1" t="str">
-        <f t="shared" ref="B4:B19" si="1">REPT("|",A4*60/MAX(A:A))</f>
+        <f t="shared" ref="B4:B23" si="1">REPT("|",A4*60/MAX(A:A))</f>
         <v>||||||||||||||||||||||||||||||||||||||||||||||||||||||||||||</v>
       </c>
       <c r="C4">
@@ -619,7 +625,7 @@
         <v>37392</v>
       </c>
       <c r="D7" s="2">
-        <f t="shared" ref="D7:D21" si="3">C6-C7</f>
+        <f t="shared" ref="D7:D24" si="3">C6-C7</f>
         <v>-16</v>
       </c>
       <c r="E7">
@@ -971,6 +977,14 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <f t="shared" ref="A20:A21" si="29">C20-$O$2</f>
+        <v>1420</v>
+      </c>
+      <c r="B20" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>|||||||||||||||</v>
+      </c>
       <c r="C20">
         <v>34188</v>
       </c>
@@ -979,11 +993,11 @@
         <v>4</v>
       </c>
       <c r="E20">
-        <f t="shared" ref="E20" si="29">$C$4-C20</f>
+        <f t="shared" ref="E20" si="30">$C$4-C20</f>
         <v>4212</v>
       </c>
       <c r="F20">
-        <f t="shared" ref="F20" si="30">$O$2-C20</f>
+        <f t="shared" ref="F20" si="31">$O$2-C20</f>
         <v>-1420</v>
       </c>
       <c r="G20" t="s">
@@ -991,6 +1005,14 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <f t="shared" si="29"/>
+        <v>1364</v>
+      </c>
+      <c r="B21" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>||||||||||||||</v>
+      </c>
       <c r="C21">
         <v>34132</v>
       </c>
@@ -999,15 +1021,71 @@
         <v>56</v>
       </c>
       <c r="E21">
-        <f t="shared" ref="E21" si="31">$C$4-C21</f>
+        <f t="shared" ref="E21" si="32">$C$4-C21</f>
         <v>4268</v>
       </c>
       <c r="F21">
-        <f t="shared" ref="F21" si="32">$O$2-C21</f>
+        <f t="shared" ref="F21" si="33">$O$2-C21</f>
         <v>-1364</v>
       </c>
       <c r="G21" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <f t="shared" ref="A22" si="34">C22-$O$2</f>
+        <v>1272</v>
+      </c>
+      <c r="B22" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>|||||||||||||</v>
+      </c>
+      <c r="C22">
+        <v>34040</v>
+      </c>
+      <c r="D22" s="2">
+        <f t="shared" si="3"/>
+        <v>92</v>
+      </c>
+      <c r="E22">
+        <f t="shared" ref="E22" si="35">$C$4-C22</f>
+        <v>4360</v>
+      </c>
+      <c r="F22">
+        <f t="shared" ref="F22" si="36">$O$2-C22</f>
+        <v>-1272</v>
+      </c>
+      <c r="G22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <f t="shared" ref="A23" si="37">C23-$O$2</f>
+        <v>1256</v>
+      </c>
+      <c r="B23" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>|||||||||||||</v>
+      </c>
+      <c r="C23">
+        <v>34024</v>
+      </c>
+      <c r="D23" s="2">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="E23">
+        <f t="shared" ref="E23" si="38">$C$4-C23</f>
+        <v>4376</v>
+      </c>
+      <c r="F23">
+        <f t="shared" ref="F23" si="39">$O$2-C23</f>
+        <v>-1256</v>
+      </c>
+      <c r="G23" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding progress output disableable notch & allpass
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC56343-A265-4828-99C2-5E0414502357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5E282D-3B79-4F2F-8025-5FAE48C47E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8640" yWindow="225" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="52995" yWindow="4020" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -109,6 +109,24 @@
   </si>
   <si>
     <t>removing uint8_t enum class, now using C++23 standard</t>
+  </si>
+  <si>
+    <t>no butterworth</t>
+  </si>
+  <si>
+    <t>minify exe player (Maj7ConsolePlayer)</t>
+  </si>
+  <si>
+    <t>re-adding butterworth and rare models</t>
+  </si>
+  <si>
+    <t>add progress reporting.</t>
+  </si>
+  <si>
+    <t>add width</t>
+  </si>
+  <si>
+    <t>remove rare models again</t>
   </si>
 </sst>
 </file>
@@ -479,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -538,7 +556,7 @@
         <v>5632</v>
       </c>
       <c r="B4" s="1" t="str">
-        <f t="shared" ref="B4:B23" si="1">REPT("|",A4*60/MAX(A:A))</f>
+        <f t="shared" ref="B4:B26" si="1">REPT("|",A4*60/MAX(A:A))</f>
         <v>||||||||||||||||||||||||||||||||||||||||||||||||||||||||||||</v>
       </c>
       <c r="C4">
@@ -625,7 +643,7 @@
         <v>37392</v>
       </c>
       <c r="D7" s="2">
-        <f t="shared" ref="D7:D24" si="3">C6-C7</f>
+        <f t="shared" ref="D7:D29" si="3">C6-C7</f>
         <v>-16</v>
       </c>
       <c r="E7">
@@ -1088,6 +1106,150 @@
         <v>27</v>
       </c>
     </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <f t="shared" ref="A24" si="40">C24-$O$2</f>
+        <v>1108</v>
+      </c>
+      <c r="B24" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>|||||||||||</v>
+      </c>
+      <c r="C24">
+        <v>33876</v>
+      </c>
+      <c r="D24" s="2">
+        <f t="shared" si="3"/>
+        <v>148</v>
+      </c>
+      <c r="E24">
+        <f t="shared" ref="E24" si="41">$C$4-C24</f>
+        <v>4524</v>
+      </c>
+      <c r="F24">
+        <f t="shared" ref="F24" si="42">$O$2-C24</f>
+        <v>-1108</v>
+      </c>
+      <c r="G24" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <f t="shared" ref="A25:A26" si="43">C25-$O$2</f>
+        <v>-428</v>
+      </c>
+      <c r="B25" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C25">
+        <v>32340</v>
+      </c>
+      <c r="D25" s="2">
+        <f t="shared" si="3"/>
+        <v>1536</v>
+      </c>
+      <c r="E25">
+        <f t="shared" ref="E25" si="44">$C$4-C25</f>
+        <v>6060</v>
+      </c>
+      <c r="F25">
+        <f t="shared" ref="F25" si="45">$O$2-C25</f>
+        <v>428</v>
+      </c>
+      <c r="G25" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <f t="shared" si="43"/>
+        <v>-132</v>
+      </c>
+      <c r="B26" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C26">
+        <v>32636</v>
+      </c>
+      <c r="D26" s="2">
+        <f t="shared" si="3"/>
+        <v>-296</v>
+      </c>
+      <c r="E26">
+        <f t="shared" ref="E26" si="46">$C$4-C26</f>
+        <v>5764</v>
+      </c>
+      <c r="F26">
+        <f t="shared" ref="F26" si="47">$O$2-C26</f>
+        <v>132</v>
+      </c>
+      <c r="G26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C27">
+        <v>32712</v>
+      </c>
+      <c r="D27" s="2">
+        <f t="shared" si="3"/>
+        <v>-76</v>
+      </c>
+      <c r="E27">
+        <f t="shared" ref="E27" si="48">$C$4-C27</f>
+        <v>5688</v>
+      </c>
+      <c r="F27">
+        <f t="shared" ref="F27" si="49">$O$2-C27</f>
+        <v>56</v>
+      </c>
+      <c r="G27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C28">
+        <v>32908</v>
+      </c>
+      <c r="D28" s="2">
+        <f t="shared" si="3"/>
+        <v>-196</v>
+      </c>
+      <c r="E28">
+        <f t="shared" ref="E28" si="50">$C$4-C28</f>
+        <v>5492</v>
+      </c>
+      <c r="F28">
+        <f t="shared" ref="F28" si="51">$O$2-C28</f>
+        <v>-140</v>
+      </c>
+      <c r="G28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C29">
+        <v>32780</v>
+      </c>
+      <c r="D29" s="2">
+        <f t="shared" si="3"/>
+        <v>128</v>
+      </c>
+      <c r="E29">
+        <f t="shared" ref="E29" si="52">$C$4-C29</f>
+        <v>5620</v>
+      </c>
+      <c r="F29">
+        <f t="shared" ref="F29" si="53">$O$2-C29</f>
+        <v>-12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
leveller Q params are now generic reso leveller now supports all filter models
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5E282D-3B79-4F2F-8025-5FAE48C47E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE44B413-6134-4A59-A572-DB61C56CFC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="52995" yWindow="4020" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>remove rare models again</t>
+  </si>
+  <si>
+    <t>remove notch &amp; allpass filter impls</t>
+  </si>
+  <si>
+    <t>tiny tweak to butterworth</t>
   </si>
 </sst>
 </file>
@@ -497,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -643,7 +649,7 @@
         <v>37392</v>
       </c>
       <c r="D7" s="2">
-        <f t="shared" ref="D7:D29" si="3">C6-C7</f>
+        <f t="shared" ref="D7:D31" si="3">C6-C7</f>
         <v>-16</v>
       </c>
       <c r="E7">
@@ -1250,6 +1256,46 @@
         <v>33</v>
       </c>
     </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C30">
+        <v>32736</v>
+      </c>
+      <c r="D30" s="2">
+        <f t="shared" si="3"/>
+        <v>44</v>
+      </c>
+      <c r="E30">
+        <f t="shared" ref="E30" si="54">$C$4-C30</f>
+        <v>5664</v>
+      </c>
+      <c r="F30">
+        <f t="shared" ref="F30" si="55">$O$2-C30</f>
+        <v>32</v>
+      </c>
+      <c r="G30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C31">
+        <v>32732</v>
+      </c>
+      <c r="D31" s="2">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="E31">
+        <f t="shared" ref="E31" si="56">$C$4-C31</f>
+        <v>5668</v>
+      </c>
+      <c r="F31">
+        <f t="shared" ref="F31" si="57">$O$2-C31</f>
+        <v>36</v>
+      </c>
+      <c r="G31" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
show command line usage fixing intrinsics breaking msvcrt again build errors in minsize rel fixing static init of luts
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBDF6358-042E-463E-9325-1C8F7A00F47D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6B60EC-E691-478C-B390-68AE21D5532F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4815" yWindow="2775" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -154,6 +154,9 @@
   </si>
   <si>
     <t>delay-based allpass, comb, delaybuffer, possibly sampler buffer could probably all share the same code</t>
+  </si>
+  <si>
+    <t>more fixing bugs, display help text</t>
   </si>
 </sst>
 </file>
@@ -524,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -1454,17 +1457,37 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C36">
+        <v>32812</v>
+      </c>
+      <c r="D36" s="2">
+        <f t="shared" ref="D36:D39" si="68">C35-C36</f>
+        <v>-4</v>
+      </c>
+      <c r="E36">
+        <f t="shared" ref="E36:E39" si="69">$C$4-C36</f>
+        <v>5588</v>
+      </c>
+      <c r="F36">
+        <f t="shared" ref="F36:F39" si="70">$O$2-C36</f>
+        <v>-44</v>
+      </c>
       <c r="G36" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G37" t="s">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G40" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G38" t="s">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removing unnecessary fn in oscillator GetModulationRecalcSampleMask to be made constexpr #121
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6B60EC-E691-478C-B390-68AE21D5532F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003CF6E5-5243-4410-9283-47484470F9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4815" yWindow="2775" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -157,6 +157,9 @@
   </si>
   <si>
     <t>more fixing bugs, display help text</t>
+  </si>
+  <si>
+    <t>removed unnecessary recalc mask</t>
   </si>
 </sst>
 </file>
@@ -1461,19 +1464,39 @@
         <v>32812</v>
       </c>
       <c r="D36" s="2">
-        <f t="shared" ref="D36:D39" si="68">C35-C36</f>
+        <f t="shared" ref="D36" si="68">C35-C36</f>
         <v>-4</v>
       </c>
       <c r="E36">
-        <f t="shared" ref="E36:E39" si="69">$C$4-C36</f>
+        <f t="shared" ref="E36" si="69">$C$4-C36</f>
         <v>5588</v>
       </c>
       <c r="F36">
-        <f t="shared" ref="F36:F39" si="70">$O$2-C36</f>
+        <f t="shared" ref="F36" si="70">$O$2-C36</f>
         <v>-44</v>
       </c>
       <c r="G36" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C37">
+        <v>32788</v>
+      </c>
+      <c r="D37" s="2">
+        <f t="shared" ref="D37" si="71">C36-C37</f>
+        <v>24</v>
+      </c>
+      <c r="E37">
+        <f t="shared" ref="E37" si="72">$C$4-C37</f>
+        <v>5612</v>
+      </c>
+      <c r="F37">
+        <f t="shared" ref="F37" si="73">$O$2-C37</f>
+        <v>-20</v>
+      </c>
+      <c r="G37" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
int and enum params now serialize in a more stable way. #128
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003CF6E5-5243-4410-9283-47484470F9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B86CB3-6117-4901-8430-7EFADC46EB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4815" yWindow="2775" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -160,6 +160,15 @@
   </si>
   <si>
     <t>removed unnecessary recalc mask</t>
+  </si>
+  <si>
+    <t>removed unnecessary lambda in oscillator ??</t>
+  </si>
+  <si>
+    <t>hardcode recalc masks</t>
+  </si>
+  <si>
+    <t>fixed int/enum serialization (core work: presets still need fixing)</t>
   </si>
 </sst>
 </file>
@@ -530,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -1499,18 +1508,78 @@
         <v>44</v>
       </c>
     </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C38">
+        <v>32768</v>
+      </c>
+      <c r="D38" s="2">
+        <f t="shared" ref="D38:D41" si="74">C37-C38</f>
+        <v>20</v>
+      </c>
+      <c r="E38">
+        <f t="shared" ref="E38:E41" si="75">$C$4-C38</f>
+        <v>5632</v>
+      </c>
+      <c r="F38">
+        <f t="shared" ref="F38:F41" si="76">$O$2-C38</f>
+        <v>0</v>
+      </c>
+      <c r="G38" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C39">
+        <v>32712</v>
+      </c>
+      <c r="D39" s="2">
+        <f t="shared" ref="D39" si="77">C38-C39</f>
+        <v>56</v>
+      </c>
+      <c r="E39">
+        <f t="shared" ref="E39" si="78">$C$4-C39</f>
+        <v>5688</v>
+      </c>
+      <c r="F39">
+        <f t="shared" ref="F39" si="79">$O$2-C39</f>
+        <v>56</v>
+      </c>
       <c r="G39" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C40">
+        <v>32656</v>
+      </c>
+      <c r="D40" s="2">
+        <f t="shared" ref="D40" si="80">C39-C40</f>
+        <v>56</v>
+      </c>
+      <c r="E40">
+        <f t="shared" ref="E40" si="81">$C$4-C40</f>
+        <v>5744</v>
+      </c>
+      <c r="F40">
+        <f t="shared" ref="F40" si="82">$O$2-C40</f>
+        <v>112</v>
+      </c>
+      <c r="G40" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G43" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G40" t="s">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G44" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G41" t="s">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G45" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
compensation gain added to oscillator level #129
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B86CB3-6117-4901-8430-7EFADC46EB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164E2B3C-9BB2-4BCE-89A6-57E8852DD845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4815" yWindow="2775" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="11100" yWindow="3060" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -169,6 +169,9 @@
   </si>
   <si>
     <t>fixed int/enum serialization (core work: presets still need fixing)</t>
+  </si>
+  <si>
+    <t>and correcting errors / defaults based on that change.</t>
   </si>
 </sst>
 </file>
@@ -1513,15 +1516,15 @@
         <v>32768</v>
       </c>
       <c r="D38" s="2">
-        <f t="shared" ref="D38:D41" si="74">C37-C38</f>
+        <f t="shared" ref="D38" si="74">C37-C38</f>
         <v>20</v>
       </c>
       <c r="E38">
-        <f t="shared" ref="E38:E41" si="75">$C$4-C38</f>
+        <f t="shared" ref="E38" si="75">$C$4-C38</f>
         <v>5632</v>
       </c>
       <c r="F38">
-        <f t="shared" ref="F38:F41" si="76">$O$2-C38</f>
+        <f t="shared" ref="F38" si="76">$O$2-C38</f>
         <v>0</v>
       </c>
       <c r="G38" t="s">
@@ -1566,6 +1569,26 @@
       </c>
       <c r="G40" t="s">
         <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C41">
+        <v>32672</v>
+      </c>
+      <c r="D41" s="2">
+        <f t="shared" ref="D41" si="83">C40-C41</f>
+        <v>-16</v>
+      </c>
+      <c r="E41">
+        <f t="shared" ref="E41" si="84">$C$4-C41</f>
+        <v>5728</v>
+      </c>
+      <c r="F41">
+        <f t="shared" ref="F41" si="85">$O$2-C41</f>
+        <v>96</v>
+      </c>
+      <c r="G41" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
now we support 4 mod envelopes
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164E2B3C-9BB2-4BCE-89A6-57E8852DD845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4839683-FAC4-4A78-BD37-AA62E4BFE446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11100" yWindow="3060" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="10755" yWindow="2715" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -172,6 +172,9 @@
   </si>
   <si>
     <t>and correcting errors / defaults based on that change.</t>
+  </si>
+  <si>
+    <t>adding 2 more mod envs</t>
   </si>
 </sst>
 </file>
@@ -542,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -1591,18 +1594,38 @@
         <v>48</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G43" t="s">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C42">
+        <v>32668</v>
+      </c>
+      <c r="D42" s="2">
+        <f t="shared" ref="D42" si="86">C41-C42</f>
+        <v>4</v>
+      </c>
+      <c r="E42">
+        <f t="shared" ref="E42" si="87">$C$4-C42</f>
+        <v>5732</v>
+      </c>
+      <c r="F42">
+        <f t="shared" ref="F42" si="88">$O$2-C42</f>
+        <v>100</v>
+      </c>
+      <c r="G42" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G46" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G44" t="s">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G47" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G45" t="s">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G48" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
alternate 0 1 mod source #101
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4839683-FAC4-4A78-BD37-AA62E4BFE446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7290C7AB-1B58-4AF2-8328-1FD64ADF72BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10755" yWindow="2715" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>adding 2 more mod envs</t>
+  </si>
+  <si>
+    <t>adding 0,1 alternating mod source</t>
   </si>
 </sst>
 </file>
@@ -1614,6 +1617,26 @@
         <v>49</v>
       </c>
     </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C43">
+        <v>32688</v>
+      </c>
+      <c r="D43" s="2">
+        <f t="shared" ref="D43" si="89">C42-C43</f>
+        <v>-20</v>
+      </c>
+      <c r="E43">
+        <f t="shared" ref="E43" si="90">$C$4-C43</f>
+        <v>5712</v>
+      </c>
+      <c r="F43">
+        <f t="shared" ref="F43" si="91">$O$2-C43</f>
+        <v>80</v>
+      </c>
+      <c r="G43" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G46" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
re-enabling pitch bend cleanup adding time basis to LFO (#71)
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7290C7AB-1B58-4AF2-8328-1FD64ADF72BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545F6317-2C6D-4501-B2F2-BE3B22A3D60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10755" yWindow="2715" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>adding 0,1 alternating mod source</t>
+  </si>
+  <si>
+    <t>enabling pitch bend</t>
   </si>
 </sst>
 </file>
@@ -1637,6 +1640,26 @@
         <v>50</v>
       </c>
     </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C44">
+        <v>32712</v>
+      </c>
+      <c r="D44" s="2">
+        <f t="shared" ref="D44" si="92">C43-C44</f>
+        <v>-24</v>
+      </c>
+      <c r="E44">
+        <f t="shared" ref="E44" si="93">$C$4-C44</f>
+        <v>5688</v>
+      </c>
+      <c r="F44">
+        <f t="shared" ref="F44" si="94">$O$2-C44</f>
+        <v>56</v>
+      </c>
+      <c r="G44" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G46" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
float serialization to json now uses bit_cast #130 int serialization to float allows more tolerance, and centers at 0 #130 adding LFO phase restart trigger #71 adding  prototype sketches of a generated param registry #131
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545F6317-2C6D-4501-B2F2-BE3B22A3D60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807C38A5-16DA-4054-8ACC-37324EF2BDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10755" yWindow="2715" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>enabling pitch bend</t>
+  </si>
+  <si>
+    <t>LFO time basis</t>
   </si>
 </sst>
 </file>
@@ -551,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -1660,18 +1663,38 @@
         <v>51</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G46" t="s">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C45">
+        <v>32824</v>
+      </c>
+      <c r="D45" s="2">
+        <f t="shared" ref="D45" si="95">C44-C45</f>
+        <v>-112</v>
+      </c>
+      <c r="E45">
+        <f t="shared" ref="E45" si="96">$C$4-C45</f>
+        <v>5576</v>
+      </c>
+      <c r="F45">
+        <f t="shared" ref="F45" si="97">$O$2-C45</f>
+        <v>-56</v>
+      </c>
+      <c r="G45" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G50" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G47" t="s">
+    <row r="51" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G51" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G48" t="s">
+    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G52" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
re-enabled stereo imager panning #135 default generation fns for all effects more refinements to int param serialization. i think it's done. #130
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807C38A5-16DA-4054-8ACC-37324EF2BDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BB2EA0-6837-4CEA-86F2-59A18FC6922C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10755" yWindow="2715" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="20475" yWindow="4230" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>LFO time basis</t>
+  </si>
+  <si>
+    <t>bit_cast int-float serialization</t>
   </si>
 </sst>
 </file>
@@ -1683,6 +1686,26 @@
         <v>52</v>
       </c>
     </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C46">
+        <v>32756</v>
+      </c>
+      <c r="D46" s="2">
+        <f t="shared" ref="D46" si="98">C45-C46</f>
+        <v>68</v>
+      </c>
+      <c r="E46">
+        <f t="shared" ref="E46" si="99">$C$4-C46</f>
+        <v>5644</v>
+      </c>
+      <c r="F46">
+        <f t="shared" ref="F46" si="100">$O$2-C46</f>
+        <v>12</v>
+      </c>
+      <c r="G46" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="50" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G50" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
adding crinkler; didn't yet get it working
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BB2EA0-6837-4CEA-86F2-59A18FC6922C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FB61C4-E1FD-4BE8-BE84-A7425D5C11A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20475" yWindow="4230" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="9585" yWindow="2340" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -187,6 +187,12 @@
   </si>
   <si>
     <t>bit_cast int-float serialization</t>
+  </si>
+  <si>
+    <t>but that isn't possible; int serialization back to unpolar. Re-enabling panning as well in width</t>
+  </si>
+  <si>
+    <t>crinkler minsizerel</t>
   </si>
 </sst>
 </file>
@@ -1447,6 +1453,14 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <f t="shared" ref="A34:A47" si="63">C34-$O$2</f>
+        <v>24</v>
+      </c>
+      <c r="B34" s="1" t="str">
+        <f t="shared" ref="B34:B47" si="64">REPT("|",A34*60/MAX(A:A))</f>
+        <v/>
+      </c>
       <c r="C34">
         <v>32792</v>
       </c>
@@ -1455,11 +1469,11 @@
         <v>72</v>
       </c>
       <c r="E34">
-        <f t="shared" ref="E34" si="63">$C$4-C34</f>
+        <f t="shared" ref="E34" si="65">$C$4-C34</f>
         <v>5608</v>
       </c>
       <c r="F34">
-        <f t="shared" ref="F34" si="64">$O$2-C34</f>
+        <f t="shared" ref="F34" si="66">$O$2-C34</f>
         <v>-24</v>
       </c>
       <c r="G34" t="s">
@@ -1467,19 +1481,27 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <f t="shared" si="63"/>
+        <v>40</v>
+      </c>
+      <c r="B35" s="1" t="str">
+        <f t="shared" si="64"/>
+        <v/>
+      </c>
       <c r="C35">
         <v>32808</v>
       </c>
       <c r="D35" s="2">
-        <f t="shared" ref="D35" si="65">C34-C35</f>
+        <f t="shared" ref="D35" si="67">C34-C35</f>
         <v>-16</v>
       </c>
       <c r="E35">
-        <f t="shared" ref="E35" si="66">$C$4-C35</f>
+        <f t="shared" ref="E35" si="68">$C$4-C35</f>
         <v>5592</v>
       </c>
       <c r="F35">
-        <f t="shared" ref="F35" si="67">$O$2-C35</f>
+        <f t="shared" ref="F35" si="69">$O$2-C35</f>
         <v>-40</v>
       </c>
       <c r="G35" t="s">
@@ -1487,19 +1509,27 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <f t="shared" si="63"/>
+        <v>44</v>
+      </c>
+      <c r="B36" s="1" t="str">
+        <f t="shared" si="64"/>
+        <v/>
+      </c>
       <c r="C36">
         <v>32812</v>
       </c>
       <c r="D36" s="2">
-        <f t="shared" ref="D36" si="68">C35-C36</f>
+        <f t="shared" ref="D36" si="70">C35-C36</f>
         <v>-4</v>
       </c>
       <c r="E36">
-        <f t="shared" ref="E36" si="69">$C$4-C36</f>
+        <f t="shared" ref="E36" si="71">$C$4-C36</f>
         <v>5588</v>
       </c>
       <c r="F36">
-        <f t="shared" ref="F36" si="70">$O$2-C36</f>
+        <f t="shared" ref="F36" si="72">$O$2-C36</f>
         <v>-44</v>
       </c>
       <c r="G36" t="s">
@@ -1507,19 +1537,27 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <f t="shared" si="63"/>
+        <v>20</v>
+      </c>
+      <c r="B37" s="1" t="str">
+        <f t="shared" si="64"/>
+        <v/>
+      </c>
       <c r="C37">
         <v>32788</v>
       </c>
       <c r="D37" s="2">
-        <f t="shared" ref="D37" si="71">C36-C37</f>
+        <f t="shared" ref="D37" si="73">C36-C37</f>
         <v>24</v>
       </c>
       <c r="E37">
-        <f t="shared" ref="E37" si="72">$C$4-C37</f>
+        <f t="shared" ref="E37" si="74">$C$4-C37</f>
         <v>5612</v>
       </c>
       <c r="F37">
-        <f t="shared" ref="F37" si="73">$O$2-C37</f>
+        <f t="shared" ref="F37" si="75">$O$2-C37</f>
         <v>-20</v>
       </c>
       <c r="G37" t="s">
@@ -1527,19 +1565,27 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <f t="shared" si="63"/>
+        <v>0</v>
+      </c>
+      <c r="B38" s="1" t="str">
+        <f t="shared" si="64"/>
+        <v/>
+      </c>
       <c r="C38">
         <v>32768</v>
       </c>
       <c r="D38" s="2">
-        <f t="shared" ref="D38" si="74">C37-C38</f>
+        <f t="shared" ref="D38" si="76">C37-C38</f>
         <v>20</v>
       </c>
       <c r="E38">
-        <f t="shared" ref="E38" si="75">$C$4-C38</f>
+        <f t="shared" ref="E38" si="77">$C$4-C38</f>
         <v>5632</v>
       </c>
       <c r="F38">
-        <f t="shared" ref="F38" si="76">$O$2-C38</f>
+        <f t="shared" ref="F38" si="78">$O$2-C38</f>
         <v>0</v>
       </c>
       <c r="G38" t="s">
@@ -1547,19 +1593,27 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <f t="shared" si="63"/>
+        <v>-56</v>
+      </c>
+      <c r="B39" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C39">
         <v>32712</v>
       </c>
       <c r="D39" s="2">
-        <f t="shared" ref="D39" si="77">C38-C39</f>
+        <f t="shared" ref="D39" si="79">C38-C39</f>
         <v>56</v>
       </c>
       <c r="E39">
-        <f t="shared" ref="E39" si="78">$C$4-C39</f>
+        <f t="shared" ref="E39" si="80">$C$4-C39</f>
         <v>5688</v>
       </c>
       <c r="F39">
-        <f t="shared" ref="F39" si="79">$O$2-C39</f>
+        <f t="shared" ref="F39" si="81">$O$2-C39</f>
         <v>56</v>
       </c>
       <c r="G39" t="s">
@@ -1567,19 +1621,27 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <f t="shared" si="63"/>
+        <v>-112</v>
+      </c>
+      <c r="B40" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C40">
         <v>32656</v>
       </c>
       <c r="D40" s="2">
-        <f t="shared" ref="D40" si="80">C39-C40</f>
+        <f t="shared" ref="D40" si="82">C39-C40</f>
         <v>56</v>
       </c>
       <c r="E40">
-        <f t="shared" ref="E40" si="81">$C$4-C40</f>
+        <f t="shared" ref="E40" si="83">$C$4-C40</f>
         <v>5744</v>
       </c>
       <c r="F40">
-        <f t="shared" ref="F40" si="82">$O$2-C40</f>
+        <f t="shared" ref="F40" si="84">$O$2-C40</f>
         <v>112</v>
       </c>
       <c r="G40" t="s">
@@ -1587,19 +1649,27 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <f t="shared" si="63"/>
+        <v>-96</v>
+      </c>
+      <c r="B41" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C41">
         <v>32672</v>
       </c>
       <c r="D41" s="2">
-        <f t="shared" ref="D41" si="83">C40-C41</f>
+        <f t="shared" ref="D41" si="85">C40-C41</f>
         <v>-16</v>
       </c>
       <c r="E41">
-        <f t="shared" ref="E41" si="84">$C$4-C41</f>
+        <f t="shared" ref="E41" si="86">$C$4-C41</f>
         <v>5728</v>
       </c>
       <c r="F41">
-        <f t="shared" ref="F41" si="85">$O$2-C41</f>
+        <f t="shared" ref="F41" si="87">$O$2-C41</f>
         <v>96</v>
       </c>
       <c r="G41" t="s">
@@ -1607,19 +1677,27 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <f t="shared" si="63"/>
+        <v>-100</v>
+      </c>
+      <c r="B42" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C42">
         <v>32668</v>
       </c>
       <c r="D42" s="2">
-        <f t="shared" ref="D42" si="86">C41-C42</f>
+        <f t="shared" ref="D42" si="88">C41-C42</f>
         <v>4</v>
       </c>
       <c r="E42">
-        <f t="shared" ref="E42" si="87">$C$4-C42</f>
+        <f t="shared" ref="E42" si="89">$C$4-C42</f>
         <v>5732</v>
       </c>
       <c r="F42">
-        <f t="shared" ref="F42" si="88">$O$2-C42</f>
+        <f t="shared" ref="F42" si="90">$O$2-C42</f>
         <v>100</v>
       </c>
       <c r="G42" t="s">
@@ -1627,19 +1705,27 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <f t="shared" si="63"/>
+        <v>-80</v>
+      </c>
+      <c r="B43" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C43">
         <v>32688</v>
       </c>
       <c r="D43" s="2">
-        <f t="shared" ref="D43" si="89">C42-C43</f>
+        <f t="shared" ref="D43" si="91">C42-C43</f>
         <v>-20</v>
       </c>
       <c r="E43">
-        <f t="shared" ref="E43" si="90">$C$4-C43</f>
+        <f t="shared" ref="E43" si="92">$C$4-C43</f>
         <v>5712</v>
       </c>
       <c r="F43">
-        <f t="shared" ref="F43" si="91">$O$2-C43</f>
+        <f t="shared" ref="F43" si="93">$O$2-C43</f>
         <v>80</v>
       </c>
       <c r="G43" t="s">
@@ -1647,19 +1733,27 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <f t="shared" si="63"/>
+        <v>-56</v>
+      </c>
+      <c r="B44" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C44">
         <v>32712</v>
       </c>
       <c r="D44" s="2">
-        <f t="shared" ref="D44" si="92">C43-C44</f>
+        <f t="shared" ref="D44" si="94">C43-C44</f>
         <v>-24</v>
       </c>
       <c r="E44">
-        <f t="shared" ref="E44" si="93">$C$4-C44</f>
+        <f t="shared" ref="E44" si="95">$C$4-C44</f>
         <v>5688</v>
       </c>
       <c r="F44">
-        <f t="shared" ref="F44" si="94">$O$2-C44</f>
+        <f t="shared" ref="F44" si="96">$O$2-C44</f>
         <v>56</v>
       </c>
       <c r="G44" t="s">
@@ -1667,19 +1761,27 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <f t="shared" si="63"/>
+        <v>56</v>
+      </c>
+      <c r="B45" s="1" t="str">
+        <f t="shared" si="64"/>
+        <v/>
+      </c>
       <c r="C45">
         <v>32824</v>
       </c>
       <c r="D45" s="2">
-        <f t="shared" ref="D45" si="95">C44-C45</f>
+        <f t="shared" ref="D45" si="97">C44-C45</f>
         <v>-112</v>
       </c>
       <c r="E45">
-        <f t="shared" ref="E45" si="96">$C$4-C45</f>
+        <f t="shared" ref="E45" si="98">$C$4-C45</f>
         <v>5576</v>
       </c>
       <c r="F45">
-        <f t="shared" ref="F45" si="97">$O$2-C45</f>
+        <f t="shared" ref="F45" si="99">$O$2-C45</f>
         <v>-56</v>
       </c>
       <c r="G45" t="s">
@@ -1687,23 +1789,64 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <f t="shared" si="63"/>
+        <v>-12</v>
+      </c>
+      <c r="B46" s="1" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C46">
         <v>32756</v>
       </c>
       <c r="D46" s="2">
-        <f t="shared" ref="D46" si="98">C45-C46</f>
+        <f t="shared" ref="D46" si="100">C45-C46</f>
         <v>68</v>
       </c>
       <c r="E46">
-        <f t="shared" ref="E46" si="99">$C$4-C46</f>
+        <f t="shared" ref="E46" si="101">$C$4-C46</f>
         <v>5644</v>
       </c>
       <c r="F46">
-        <f t="shared" ref="F46" si="100">$O$2-C46</f>
+        <f t="shared" ref="F46" si="102">$O$2-C46</f>
         <v>12</v>
       </c>
       <c r="G46" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <f t="shared" si="63"/>
+        <v>36</v>
+      </c>
+      <c r="B47" s="1" t="str">
+        <f t="shared" si="64"/>
+        <v/>
+      </c>
+      <c r="C47">
+        <v>32804</v>
+      </c>
+      <c r="D47" s="2">
+        <f t="shared" ref="D47" si="103">C46-C47</f>
+        <v>-48</v>
+      </c>
+      <c r="E47">
+        <f t="shared" ref="E47" si="104">$C$4-C47</f>
+        <v>5596</v>
+      </c>
+      <c r="F47">
+        <f t="shared" ref="F47" si="105">$O$2-C47</f>
+        <v>-36</v>
+      </c>
+      <c r="G47" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G48" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="50" spans="7:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
#133 fixing new defaults with -1..1 int and floatn11 param storage
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FB61C4-E1FD-4BE8-BE84-A7425D5C11A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719BC422-D260-4FC1-9426-88D24932FF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9585" yWindow="2340" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -192,7 +192,7 @@
     <t>but that isn't possible; int serialization back to unpolar. Re-enabling panning as well in width</t>
   </si>
   <si>
-    <t>crinkler minsizerel</t>
+    <t>#133 using -1..1 floats for defaults</t>
   </si>
 </sst>
 </file>
@@ -563,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
@@ -1845,22 +1845,37 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C48">
+        <v>32744</v>
+      </c>
+      <c r="D48" s="2">
+        <f t="shared" ref="D48" si="106">C47-C48</f>
+        <v>60</v>
+      </c>
+      <c r="E48">
+        <f t="shared" ref="E48" si="107">$C$4-C48</f>
+        <v>5656</v>
+      </c>
+      <c r="F48">
+        <f t="shared" ref="F48" si="108">$O$2-C48</f>
+        <v>24</v>
+      </c>
       <c r="G48" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G50" t="s">
+    <row r="54" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G54" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G51" t="s">
+    <row r="55" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G55" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G52" t="s">
+    <row r="56" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G56" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
- unifying delay/comb/allpass/audio buffers - pod vector
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719BC422-D260-4FC1-9426-88D24932FF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCA5054-995C-4AB3-AD04-D59162281754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9585" yWindow="2340" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -147,15 +147,6 @@
     <t>massive refactor</t>
   </si>
   <si>
-    <t>TODO opportunities:</t>
-  </si>
-  <si>
-    <t>driverEnumCallback</t>
-  </si>
-  <si>
-    <t>delay-based allpass, comb, delaybuffer, possibly sampler buffer could probably all share the same code</t>
-  </si>
-  <si>
     <t>more fixing bugs, display help text</t>
   </si>
   <si>
@@ -193,6 +184,24 @@
   </si>
   <si>
     <t>#133 using -1..1 floats for defaults</t>
+  </si>
+  <si>
+    <t>#137 value noise fbm</t>
+  </si>
+  <si>
+    <t>no noise inlines</t>
+  </si>
+  <si>
+    <t>cheaper noise</t>
+  </si>
+  <si>
+    <t>remove FBM option</t>
+  </si>
+  <si>
+    <t>podvector to replace various  buffers</t>
+  </si>
+  <si>
+    <t>better ctor, various optimizations, unifying allpass, delay, comb, audiobuffers</t>
   </si>
 </sst>
 </file>
@@ -563,10 +572,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="45" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="6" customWidth="1"/>
@@ -603,8 +612,8 @@
         <v>5120</v>
       </c>
       <c r="B3" s="1" t="str">
-        <f>REPT("|",A3*60/MAX(A:A))</f>
-        <v>||||||||||||||||||||||||||||||||||||||||||||||||||||||</v>
+        <f>REPT("#",A3*100/MAX(A:A))</f>
+        <v>##########################################################################################</v>
       </c>
       <c r="C3">
         <v>37888</v>
@@ -622,8 +631,8 @@
         <v>5632</v>
       </c>
       <c r="B4" s="1" t="str">
-        <f t="shared" ref="B4:B33" si="1">REPT("|",A4*60/MAX(A:A))</f>
-        <v>||||||||||||||||||||||||||||||||||||||||||||||||||||||||||||</v>
+        <f t="shared" ref="B4:B54" si="1">REPT("#",A4*100/MAX(A:A))</f>
+        <v>####################################################################################################</v>
       </c>
       <c r="C4">
         <v>38400</v>
@@ -647,7 +656,7 @@
       </c>
       <c r="B5" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||||||||||||||||||||||||||||||||||||||||||</v>
+        <v>##########################################################################################</v>
       </c>
       <c r="C5">
         <v>37888</v>
@@ -675,7 +684,7 @@
       </c>
       <c r="B6" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||||||||||||||||||</v>
+        <v>#################################################################################</v>
       </c>
       <c r="C6">
         <v>37376</v>
@@ -703,7 +712,7 @@
       </c>
       <c r="B7" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||||||||||||||||||</v>
+        <v>##################################################################################</v>
       </c>
       <c r="C7">
         <v>37392</v>
@@ -731,7 +740,7 @@
       </c>
       <c r="B8" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||||||||||</v>
+        <v>####################################################################</v>
       </c>
       <c r="C8">
         <v>36636</v>
@@ -759,7 +768,7 @@
       </c>
       <c r="B9" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||||||||||</v>
+        <v>####################################################################</v>
       </c>
       <c r="C9">
         <v>36624</v>
@@ -787,7 +796,7 @@
       </c>
       <c r="B10" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||||||||||</v>
+        <v>####################################################################</v>
       </c>
       <c r="C10">
         <v>36632</v>
@@ -815,7 +824,7 @@
       </c>
       <c r="B11" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||||||||||</v>
+        <v>####################################################################</v>
       </c>
       <c r="C11">
         <v>36648</v>
@@ -843,7 +852,7 @@
       </c>
       <c r="B12" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||||||||||||||||||||</v>
+        <v>#######################################################</v>
       </c>
       <c r="C12">
         <v>35920</v>
@@ -871,7 +880,7 @@
       </c>
       <c r="B13" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||||||||||||||||||||</v>
+        <v>######################################################</v>
       </c>
       <c r="C13">
         <v>35844</v>
@@ -899,7 +908,7 @@
       </c>
       <c r="B14" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||||||||||||||||||||</v>
+        <v>######################################################</v>
       </c>
       <c r="C14">
         <v>35836</v>
@@ -927,7 +936,7 @@
       </c>
       <c r="B15" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||||||||||||||||||</v>
+        <v>##################################################</v>
       </c>
       <c r="C15">
         <v>35592</v>
@@ -955,7 +964,7 @@
       </c>
       <c r="B16" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||</v>
+        <v>#########################</v>
       </c>
       <c r="C16">
         <v>34220</v>
@@ -983,7 +992,7 @@
       </c>
       <c r="B17" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||||</v>
+        <v>##########################</v>
       </c>
       <c r="C17">
         <v>34280</v>
@@ -1011,7 +1020,7 @@
       </c>
       <c r="B18" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||||</v>
+        <v>##########################</v>
       </c>
       <c r="C18">
         <v>34276</v>
@@ -1039,7 +1048,7 @@
       </c>
       <c r="B19" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||</v>
+        <v>#########################</v>
       </c>
       <c r="C19">
         <v>34192</v>
@@ -1067,7 +1076,7 @@
       </c>
       <c r="B20" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||||</v>
+        <v>#########################</v>
       </c>
       <c r="C20">
         <v>34188</v>
@@ -1095,7 +1104,7 @@
       </c>
       <c r="B21" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>||||||||||||||</v>
+        <v>########################</v>
       </c>
       <c r="C21">
         <v>34132</v>
@@ -1123,7 +1132,7 @@
       </c>
       <c r="B22" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||</v>
+        <v>######################</v>
       </c>
       <c r="C22">
         <v>34040</v>
@@ -1151,7 +1160,7 @@
       </c>
       <c r="B23" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||||</v>
+        <v>######################</v>
       </c>
       <c r="C23">
         <v>34024</v>
@@ -1179,7 +1188,7 @@
       </c>
       <c r="B24" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|||||||||||</v>
+        <v>###################</v>
       </c>
       <c r="C24">
         <v>33876</v>
@@ -1291,7 +1300,7 @@
       </c>
       <c r="B28" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|</v>
+        <v>##</v>
       </c>
       <c r="C28">
         <v>32908</v>
@@ -1431,7 +1440,7 @@
       </c>
       <c r="B33" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>|</v>
+        <v>#</v>
       </c>
       <c r="C33">
         <v>32864</v>
@@ -1458,7 +1467,7 @@
         <v>24</v>
       </c>
       <c r="B34" s="1" t="str">
-        <f t="shared" ref="B34:B47" si="64">REPT("|",A34*60/MAX(A:A))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C34">
@@ -1469,11 +1478,11 @@
         <v>72</v>
       </c>
       <c r="E34">
-        <f t="shared" ref="E34" si="65">$C$4-C34</f>
+        <f t="shared" ref="E34" si="64">$C$4-C34</f>
         <v>5608</v>
       </c>
       <c r="F34">
-        <f t="shared" ref="F34" si="66">$O$2-C34</f>
+        <f t="shared" ref="F34" si="65">$O$2-C34</f>
         <v>-24</v>
       </c>
       <c r="G34" t="s">
@@ -1486,22 +1495,22 @@
         <v>40</v>
       </c>
       <c r="B35" s="1" t="str">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C35">
         <v>32808</v>
       </c>
       <c r="D35" s="2">
-        <f t="shared" ref="D35" si="67">C34-C35</f>
+        <f t="shared" ref="D35" si="66">C34-C35</f>
         <v>-16</v>
       </c>
       <c r="E35">
-        <f t="shared" ref="E35" si="68">$C$4-C35</f>
+        <f t="shared" ref="E35" si="67">$C$4-C35</f>
         <v>5592</v>
       </c>
       <c r="F35">
-        <f t="shared" ref="F35" si="69">$O$2-C35</f>
+        <f t="shared" ref="F35" si="68">$O$2-C35</f>
         <v>-40</v>
       </c>
       <c r="G35" t="s">
@@ -1514,26 +1523,26 @@
         <v>44</v>
       </c>
       <c r="B36" s="1" t="str">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C36">
         <v>32812</v>
       </c>
       <c r="D36" s="2">
-        <f t="shared" ref="D36" si="70">C35-C36</f>
+        <f t="shared" ref="D36" si="69">C35-C36</f>
         <v>-4</v>
       </c>
       <c r="E36">
-        <f t="shared" ref="E36" si="71">$C$4-C36</f>
+        <f t="shared" ref="E36" si="70">$C$4-C36</f>
         <v>5588</v>
       </c>
       <c r="F36">
-        <f t="shared" ref="F36" si="72">$O$2-C36</f>
+        <f t="shared" ref="F36" si="71">$O$2-C36</f>
         <v>-44</v>
       </c>
       <c r="G36" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -1542,26 +1551,26 @@
         <v>20</v>
       </c>
       <c r="B37" s="1" t="str">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C37">
         <v>32788</v>
       </c>
       <c r="D37" s="2">
-        <f t="shared" ref="D37" si="73">C36-C37</f>
+        <f t="shared" ref="D37" si="72">C36-C37</f>
         <v>24</v>
       </c>
       <c r="E37">
-        <f t="shared" ref="E37" si="74">$C$4-C37</f>
+        <f t="shared" ref="E37" si="73">$C$4-C37</f>
         <v>5612</v>
       </c>
       <c r="F37">
-        <f t="shared" ref="F37" si="75">$O$2-C37</f>
+        <f t="shared" ref="F37" si="74">$O$2-C37</f>
         <v>-20</v>
       </c>
       <c r="G37" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -1570,26 +1579,26 @@
         <v>0</v>
       </c>
       <c r="B38" s="1" t="str">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C38">
         <v>32768</v>
       </c>
       <c r="D38" s="2">
-        <f t="shared" ref="D38" si="76">C37-C38</f>
+        <f t="shared" ref="D38" si="75">C37-C38</f>
         <v>20</v>
       </c>
       <c r="E38">
-        <f t="shared" ref="E38" si="77">$C$4-C38</f>
+        <f t="shared" ref="E38" si="76">$C$4-C38</f>
         <v>5632</v>
       </c>
       <c r="F38">
-        <f t="shared" ref="F38" si="78">$O$2-C38</f>
+        <f t="shared" ref="F38" si="77">$O$2-C38</f>
         <v>0</v>
       </c>
       <c r="G38" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1598,26 +1607,26 @@
         <v>-56</v>
       </c>
       <c r="B39" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C39">
         <v>32712</v>
       </c>
       <c r="D39" s="2">
-        <f t="shared" ref="D39" si="79">C38-C39</f>
+        <f t="shared" ref="D39" si="78">C38-C39</f>
         <v>56</v>
       </c>
       <c r="E39">
-        <f t="shared" ref="E39" si="80">$C$4-C39</f>
+        <f t="shared" ref="E39" si="79">$C$4-C39</f>
         <v>5688</v>
       </c>
       <c r="F39">
-        <f t="shared" ref="F39" si="81">$O$2-C39</f>
+        <f t="shared" ref="F39" si="80">$O$2-C39</f>
         <v>56</v>
       </c>
       <c r="G39" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -1626,26 +1635,26 @@
         <v>-112</v>
       </c>
       <c r="B40" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C40">
         <v>32656</v>
       </c>
       <c r="D40" s="2">
-        <f t="shared" ref="D40" si="82">C39-C40</f>
+        <f t="shared" ref="D40" si="81">C39-C40</f>
         <v>56</v>
       </c>
       <c r="E40">
-        <f t="shared" ref="E40" si="83">$C$4-C40</f>
+        <f t="shared" ref="E40" si="82">$C$4-C40</f>
         <v>5744</v>
       </c>
       <c r="F40">
-        <f t="shared" ref="F40" si="84">$O$2-C40</f>
+        <f t="shared" ref="F40" si="83">$O$2-C40</f>
         <v>112</v>
       </c>
       <c r="G40" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -1654,26 +1663,26 @@
         <v>-96</v>
       </c>
       <c r="B41" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C41">
         <v>32672</v>
       </c>
       <c r="D41" s="2">
-        <f t="shared" ref="D41" si="85">C40-C41</f>
+        <f t="shared" ref="D41" si="84">C40-C41</f>
         <v>-16</v>
       </c>
       <c r="E41">
-        <f t="shared" ref="E41" si="86">$C$4-C41</f>
+        <f t="shared" ref="E41" si="85">$C$4-C41</f>
         <v>5728</v>
       </c>
       <c r="F41">
-        <f t="shared" ref="F41" si="87">$O$2-C41</f>
+        <f t="shared" ref="F41" si="86">$O$2-C41</f>
         <v>96</v>
       </c>
       <c r="G41" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -1682,26 +1691,26 @@
         <v>-100</v>
       </c>
       <c r="B42" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C42">
         <v>32668</v>
       </c>
       <c r="D42" s="2">
-        <f t="shared" ref="D42" si="88">C41-C42</f>
+        <f t="shared" ref="D42" si="87">C41-C42</f>
         <v>4</v>
       </c>
       <c r="E42">
-        <f t="shared" ref="E42" si="89">$C$4-C42</f>
+        <f t="shared" ref="E42" si="88">$C$4-C42</f>
         <v>5732</v>
       </c>
       <c r="F42">
-        <f t="shared" ref="F42" si="90">$O$2-C42</f>
+        <f t="shared" ref="F42" si="89">$O$2-C42</f>
         <v>100</v>
       </c>
       <c r="G42" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -1710,26 +1719,26 @@
         <v>-80</v>
       </c>
       <c r="B43" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C43">
         <v>32688</v>
       </c>
       <c r="D43" s="2">
-        <f t="shared" ref="D43" si="91">C42-C43</f>
+        <f t="shared" ref="D43" si="90">C42-C43</f>
         <v>-20</v>
       </c>
       <c r="E43">
-        <f t="shared" ref="E43" si="92">$C$4-C43</f>
+        <f t="shared" ref="E43" si="91">$C$4-C43</f>
         <v>5712</v>
       </c>
       <c r="F43">
-        <f t="shared" ref="F43" si="93">$O$2-C43</f>
+        <f t="shared" ref="F43" si="92">$O$2-C43</f>
         <v>80</v>
       </c>
       <c r="G43" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -1738,26 +1747,26 @@
         <v>-56</v>
       </c>
       <c r="B44" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C44">
         <v>32712</v>
       </c>
       <c r="D44" s="2">
-        <f t="shared" ref="D44" si="94">C43-C44</f>
+        <f t="shared" ref="D44" si="93">C43-C44</f>
         <v>-24</v>
       </c>
       <c r="E44">
-        <f t="shared" ref="E44" si="95">$C$4-C44</f>
+        <f t="shared" ref="E44" si="94">$C$4-C44</f>
         <v>5688</v>
       </c>
       <c r="F44">
-        <f t="shared" ref="F44" si="96">$O$2-C44</f>
+        <f t="shared" ref="F44" si="95">$O$2-C44</f>
         <v>56</v>
       </c>
       <c r="G44" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -1766,26 +1775,26 @@
         <v>56</v>
       </c>
       <c r="B45" s="1" t="str">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C45">
         <v>32824</v>
       </c>
       <c r="D45" s="2">
-        <f t="shared" ref="D45" si="97">C44-C45</f>
+        <f t="shared" ref="D45" si="96">C44-C45</f>
         <v>-112</v>
       </c>
       <c r="E45">
-        <f t="shared" ref="E45" si="98">$C$4-C45</f>
+        <f t="shared" ref="E45" si="97">$C$4-C45</f>
         <v>5576</v>
       </c>
       <c r="F45">
-        <f t="shared" ref="F45" si="99">$O$2-C45</f>
+        <f t="shared" ref="F45" si="98">$O$2-C45</f>
         <v>-56</v>
       </c>
       <c r="G45" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -1794,26 +1803,26 @@
         <v>-12</v>
       </c>
       <c r="B46" s="1" t="e">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
       <c r="C46">
         <v>32756</v>
       </c>
       <c r="D46" s="2">
-        <f t="shared" ref="D46" si="100">C45-C46</f>
+        <f t="shared" ref="D46" si="99">C45-C46</f>
         <v>68</v>
       </c>
       <c r="E46">
-        <f t="shared" ref="E46" si="101">$C$4-C46</f>
+        <f t="shared" ref="E46" si="100">$C$4-C46</f>
         <v>5644</v>
       </c>
       <c r="F46">
-        <f t="shared" ref="F46" si="102">$O$2-C46</f>
+        <f t="shared" ref="F46" si="101">$O$2-C46</f>
         <v>12</v>
       </c>
       <c r="G46" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -1822,29 +1831,37 @@
         <v>36</v>
       </c>
       <c r="B47" s="1" t="str">
-        <f t="shared" si="64"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="C47">
         <v>32804</v>
       </c>
       <c r="D47" s="2">
-        <f t="shared" ref="D47" si="103">C46-C47</f>
+        <f t="shared" ref="D47" si="102">C46-C47</f>
         <v>-48</v>
       </c>
       <c r="E47">
-        <f t="shared" ref="E47" si="104">$C$4-C47</f>
+        <f t="shared" ref="E47" si="103">$C$4-C47</f>
         <v>5596</v>
       </c>
       <c r="F47">
-        <f t="shared" ref="F47" si="105">$O$2-C47</f>
+        <f t="shared" ref="F47" si="104">$O$2-C47</f>
         <v>-36</v>
       </c>
       <c r="G47" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <f t="shared" ref="A48:A54" si="105">C48-$O$2</f>
+        <v>-24</v>
+      </c>
+      <c r="B48" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C48">
         <v>32744</v>
       </c>
@@ -1861,22 +1878,175 @@
         <v>24</v>
       </c>
       <c r="G48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <f t="shared" si="105"/>
+        <v>344</v>
+      </c>
+      <c r="B49" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>######</v>
+      </c>
+      <c r="C49">
+        <v>33112</v>
+      </c>
+      <c r="D49" s="2">
+        <f t="shared" ref="D49" si="109">C48-C49</f>
+        <v>-368</v>
+      </c>
+      <c r="E49">
+        <f t="shared" ref="E49" si="110">$C$4-C49</f>
+        <v>5288</v>
+      </c>
+      <c r="F49">
+        <f t="shared" ref="F49" si="111">$O$2-C49</f>
+        <v>-344</v>
+      </c>
+      <c r="G49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <f t="shared" si="105"/>
+        <v>340</v>
+      </c>
+      <c r="B50" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>######</v>
+      </c>
+      <c r="C50">
+        <v>33108</v>
+      </c>
+      <c r="D50" s="2">
+        <f t="shared" ref="D50" si="112">C49-C50</f>
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <f t="shared" ref="E50" si="113">$C$4-C50</f>
+        <v>5292</v>
+      </c>
+      <c r="F50">
+        <f t="shared" ref="F50" si="114">$O$2-C50</f>
+        <v>-340</v>
+      </c>
+      <c r="G50" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <f t="shared" si="105"/>
+        <v>296</v>
+      </c>
+      <c r="B51" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>#####</v>
+      </c>
+      <c r="C51">
+        <v>33064</v>
+      </c>
+      <c r="D51" s="2">
+        <f t="shared" ref="D51" si="115">C50-C51</f>
+        <v>44</v>
+      </c>
+      <c r="E51">
+        <f t="shared" ref="E51" si="116">$C$4-C51</f>
+        <v>5336</v>
+      </c>
+      <c r="F51">
+        <f t="shared" ref="F51" si="117">$O$2-C51</f>
+        <v>-296</v>
+      </c>
+      <c r="G51" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="54" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <f t="shared" si="105"/>
+        <v>256</v>
+      </c>
+      <c r="B52" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>####</v>
+      </c>
+      <c r="C52">
+        <v>33024</v>
+      </c>
+      <c r="D52" s="2">
+        <f t="shared" ref="D52" si="118">C51-C52</f>
+        <v>40</v>
+      </c>
+      <c r="E52">
+        <f t="shared" ref="E52" si="119">$C$4-C52</f>
+        <v>5376</v>
+      </c>
+      <c r="F52">
+        <f t="shared" ref="F52" si="120">$O$2-C52</f>
+        <v>-256</v>
+      </c>
+      <c r="G52" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <f t="shared" si="105"/>
+        <v>424</v>
+      </c>
+      <c r="B53" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>#######</v>
+      </c>
+      <c r="C53">
+        <v>33192</v>
+      </c>
+      <c r="D53" s="2">
+        <f t="shared" ref="D53" si="121">C52-C53</f>
+        <v>-168</v>
+      </c>
+      <c r="E53">
+        <f t="shared" ref="E53" si="122">$C$4-C53</f>
+        <v>5208</v>
+      </c>
+      <c r="F53">
+        <f t="shared" ref="F53" si="123">$O$2-C53</f>
+        <v>-424</v>
+      </c>
+      <c r="G53" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <f t="shared" si="105"/>
+        <v>264</v>
+      </c>
+      <c r="B54" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>####</v>
+      </c>
+      <c r="C54">
+        <v>33032</v>
+      </c>
+      <c r="D54" s="2">
+        <f t="shared" ref="D54" si="124">C53-C54</f>
+        <v>160</v>
+      </c>
+      <c r="E54">
+        <f t="shared" ref="E54" si="125">$C$4-C54</f>
+        <v>5368</v>
+      </c>
+      <c r="F54">
+        <f t="shared" ref="F54" si="126">$O$2-C54</f>
+        <v>-264</v>
+      </c>
       <c r="G54" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="55" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G55" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="56" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G56" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removing sample interpolation option hard-removing GSM support to save bits and allow simpler ownership/object lifetimes #138
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCA5054-995C-4AB3-AD04-D59162281754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7033B1-F036-46EB-B08A-278457666247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -202,6 +202,12 @@
   </si>
   <si>
     <t>better ctor, various optimizations, unifying allpass, delay, comb, audiobuffers</t>
+  </si>
+  <si>
+    <t>remove interpolation mode, sampler optimizations</t>
+  </si>
+  <si>
+    <t>gmdls is now the only sample source</t>
   </si>
 </sst>
 </file>
@@ -572,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -631,7 +637,7 @@
         <v>5632</v>
       </c>
       <c r="B4" s="1" t="str">
-        <f t="shared" ref="B4:B54" si="1">REPT("#",A4*100/MAX(A:A))</f>
+        <f t="shared" ref="B4:B56" si="1">REPT("#",A4*100/MAX(A:A))</f>
         <v>####################################################################################################</v>
       </c>
       <c r="C4">
@@ -2024,29 +2030,85 @@
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54">
         <f t="shared" si="105"/>
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="B54" s="1" t="str">
         <f t="shared" si="1"/>
         <v>####</v>
       </c>
       <c r="C54">
-        <v>33032</v>
+        <v>33024</v>
       </c>
       <c r="D54" s="2">
         <f t="shared" ref="D54" si="124">C53-C54</f>
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E54">
         <f t="shared" ref="E54" si="125">$C$4-C54</f>
-        <v>5368</v>
+        <v>5376</v>
       </c>
       <c r="F54">
         <f t="shared" ref="F54" si="126">$O$2-C54</f>
-        <v>-264</v>
+        <v>-256</v>
       </c>
       <c r="G54" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <f t="shared" ref="A55:A56" si="127">C55-$O$2</f>
+        <v>232</v>
+      </c>
+      <c r="B55" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>####</v>
+      </c>
+      <c r="C55">
+        <v>33000</v>
+      </c>
+      <c r="D55" s="2">
+        <f t="shared" ref="D55" si="128">C54-C55</f>
+        <v>24</v>
+      </c>
+      <c r="E55">
+        <f t="shared" ref="E55" si="129">$C$4-C55</f>
+        <v>5400</v>
+      </c>
+      <c r="F55">
+        <f t="shared" ref="F55" si="130">$O$2-C55</f>
+        <v>-232</v>
+      </c>
+      <c r="G55" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <f t="shared" si="127"/>
+        <v>156</v>
+      </c>
+      <c r="B56" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>##</v>
+      </c>
+      <c r="C56">
+        <v>32924</v>
+      </c>
+      <c r="D56" s="2">
+        <f t="shared" ref="D56" si="131">C55-C56</f>
+        <v>76</v>
+      </c>
+      <c r="E56">
+        <f t="shared" ref="E56" si="132">$C$4-C56</f>
+        <v>5476</v>
+      </c>
+      <c r="F56">
+        <f t="shared" ref="F56" si="133">$O$2-C56</f>
+        <v>-156</v>
+      </c>
+      <c r="G56" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed #150: envelope curve params
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{400DAB32-84A4-4628-9038-3F69F1C3BF51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47FF6D7-E630-4708-8BD2-25D9B4027FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -220,6 +220,9 @@
   </si>
   <si>
     <t>disable pulse4</t>
+  </si>
+  <si>
+    <t>fix to precision for rotating noise #144</t>
   </si>
 </sst>
 </file>
@@ -590,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2235,6 +2238,43 @@
         <v>64</v>
       </c>
     </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C61">
+        <v>32924</v>
+      </c>
+      <c r="D61" s="2">
+        <f t="shared" ref="D61" si="149">C60-C61</f>
+        <v>-84</v>
+      </c>
+      <c r="E61">
+        <f t="shared" ref="E61" si="150">$C$4-C61</f>
+        <v>5476</v>
+      </c>
+      <c r="F61">
+        <f t="shared" ref="F61" si="151">$O$2-C61</f>
+        <v>-156</v>
+      </c>
+      <c r="G61" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C62">
+        <v>32924</v>
+      </c>
+      <c r="D62" s="2">
+        <f t="shared" ref="D62" si="152">C61-C62</f>
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <f t="shared" ref="E62" si="153">$C$4-C62</f>
+        <v>5476</v>
+      </c>
+      <c r="F62">
+        <f t="shared" ref="F62" si="154">$O$2-C62</f>
+        <v>-156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
#152 WIP removing 6db/oct option entirely; too complex and not useful simplifications, revisions....
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47FF6D7-E630-4708-8BD2-25D9B4027FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0573EFD5-99BE-4A4D-991B-8B046B4C338F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -223,6 +223,18 @@
   </si>
   <si>
     <t>fix to precision for rotating noise #144</t>
+  </si>
+  <si>
+    <t>mbc fixes #151</t>
+  </si>
+  <si>
+    <t>re-enabling crossover slopes-adding params and infra</t>
+  </si>
+  <si>
+    <t>impl naïve</t>
+  </si>
+  <si>
+    <t>removing a bunch of unnecessary bloat</t>
   </si>
 </sst>
 </file>
@@ -593,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2260,19 +2272,82 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C62">
-        <v>32924</v>
+        <v>32964</v>
       </c>
       <c r="D62" s="2">
         <f t="shared" ref="D62" si="152">C61-C62</f>
-        <v>0</v>
+        <v>-40</v>
       </c>
       <c r="E62">
         <f t="shared" ref="E62" si="153">$C$4-C62</f>
-        <v>5476</v>
+        <v>5436</v>
       </c>
       <c r="F62">
         <f t="shared" ref="F62" si="154">$O$2-C62</f>
-        <v>-156</v>
+        <v>-196</v>
+      </c>
+      <c r="G62" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C63">
+        <v>32884</v>
+      </c>
+      <c r="D63" s="2">
+        <f t="shared" ref="D63" si="155">C62-C63</f>
+        <v>80</v>
+      </c>
+      <c r="E63">
+        <f t="shared" ref="E63" si="156">$C$4-C63</f>
+        <v>5516</v>
+      </c>
+      <c r="F63">
+        <f t="shared" ref="F63" si="157">$O$2-C63</f>
+        <v>-116</v>
+      </c>
+      <c r="G63" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C64">
+        <v>33408</v>
+      </c>
+      <c r="D64" s="2">
+        <f t="shared" ref="D64" si="158">C63-C64</f>
+        <v>-524</v>
+      </c>
+      <c r="E64">
+        <f t="shared" ref="E64" si="159">$C$4-C64</f>
+        <v>4992</v>
+      </c>
+      <c r="F64">
+        <f t="shared" ref="F64" si="160">$O$2-C64</f>
+        <v>-640</v>
+      </c>
+      <c r="G64" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C65">
+        <v>33216</v>
+      </c>
+      <c r="D65" s="2">
+        <f t="shared" ref="D65" si="161">C64-C65</f>
+        <v>192</v>
+      </c>
+      <c r="E65">
+        <f t="shared" ref="E65" si="162">$C$4-C65</f>
+        <v>5184</v>
+      </c>
+      <c r="F65">
+        <f t="shared" ref="F65" si="163">$O$2-C65</f>
+        <v>-448</v>
+      </c>
+      <c r="G65" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed more mbc volume issues with soft clipper
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0573EFD5-99BE-4A4D-991B-8B046B4C338F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E862B35-6986-4B46-911A-7CE0907CFB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -235,6 +235,18 @@
   </si>
   <si>
     <t>removing a bunch of unnecessary bloat</t>
+  </si>
+  <si>
+    <t>removing model gain compensation for mbc</t>
+  </si>
+  <si>
+    <t>gating out 12 and 36db/oct crossovers</t>
+  </si>
+  <si>
+    <t>single crossover option, optimizations</t>
+  </si>
+  <si>
+    <t>de-inlining moog one pole filter</t>
   </si>
 </sst>
 </file>
@@ -605,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2251,19 +2263,27 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <f t="shared" ref="A61:A65" si="149">C61-$O$2</f>
+        <v>156</v>
+      </c>
+      <c r="B61" s="1" t="str">
+        <f t="shared" ref="B61:B65" si="150">REPT("#",A61*100/MAX(A:A))</f>
+        <v>##</v>
+      </c>
       <c r="C61">
         <v>32924</v>
       </c>
       <c r="D61" s="2">
-        <f t="shared" ref="D61" si="149">C60-C61</f>
+        <f t="shared" ref="D61" si="151">C60-C61</f>
         <v>-84</v>
       </c>
       <c r="E61">
-        <f t="shared" ref="E61" si="150">$C$4-C61</f>
+        <f t="shared" ref="E61" si="152">$C$4-C61</f>
         <v>5476</v>
       </c>
       <c r="F61">
-        <f t="shared" ref="F61" si="151">$O$2-C61</f>
+        <f t="shared" ref="F61" si="153">$O$2-C61</f>
         <v>-156</v>
       </c>
       <c r="G61" t="s">
@@ -2271,19 +2291,27 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <f t="shared" si="149"/>
+        <v>196</v>
+      </c>
+      <c r="B62" s="1" t="str">
+        <f t="shared" si="150"/>
+        <v>###</v>
+      </c>
       <c r="C62">
         <v>32964</v>
       </c>
       <c r="D62" s="2">
-        <f t="shared" ref="D62" si="152">C61-C62</f>
+        <f t="shared" ref="D62" si="154">C61-C62</f>
         <v>-40</v>
       </c>
       <c r="E62">
-        <f t="shared" ref="E62" si="153">$C$4-C62</f>
+        <f t="shared" ref="E62" si="155">$C$4-C62</f>
         <v>5436</v>
       </c>
       <c r="F62">
-        <f t="shared" ref="F62" si="154">$O$2-C62</f>
+        <f t="shared" ref="F62" si="156">$O$2-C62</f>
         <v>-196</v>
       </c>
       <c r="G62" t="s">
@@ -2291,19 +2319,27 @@
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <f t="shared" si="149"/>
+        <v>116</v>
+      </c>
+      <c r="B63" s="1" t="str">
+        <f t="shared" si="150"/>
+        <v>##</v>
+      </c>
       <c r="C63">
         <v>32884</v>
       </c>
       <c r="D63" s="2">
-        <f t="shared" ref="D63" si="155">C62-C63</f>
+        <f t="shared" ref="D63" si="157">C62-C63</f>
         <v>80</v>
       </c>
       <c r="E63">
-        <f t="shared" ref="E63" si="156">$C$4-C63</f>
+        <f t="shared" ref="E63" si="158">$C$4-C63</f>
         <v>5516</v>
       </c>
       <c r="F63">
-        <f t="shared" ref="F63" si="157">$O$2-C63</f>
+        <f t="shared" ref="F63" si="159">$O$2-C63</f>
         <v>-116</v>
       </c>
       <c r="G63" t="s">
@@ -2311,43 +2347,139 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <f t="shared" si="149"/>
+        <v>640</v>
+      </c>
+      <c r="B64" s="1" t="str">
+        <f t="shared" si="150"/>
+        <v>###########</v>
+      </c>
       <c r="C64">
         <v>33408</v>
       </c>
       <c r="D64" s="2">
-        <f t="shared" ref="D64" si="158">C63-C64</f>
+        <f t="shared" ref="D64" si="160">C63-C64</f>
         <v>-524</v>
       </c>
       <c r="E64">
-        <f t="shared" ref="E64" si="159">$C$4-C64</f>
+        <f t="shared" ref="E64" si="161">$C$4-C64</f>
         <v>4992</v>
       </c>
       <c r="F64">
-        <f t="shared" ref="F64" si="160">$O$2-C64</f>
+        <f t="shared" ref="F64" si="162">$O$2-C64</f>
         <v>-640</v>
       </c>
       <c r="G64" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <f t="shared" si="149"/>
+        <v>440</v>
+      </c>
+      <c r="B65" s="1" t="str">
+        <f t="shared" si="150"/>
+        <v>#######</v>
+      </c>
       <c r="C65">
-        <v>33216</v>
+        <v>33208</v>
       </c>
       <c r="D65" s="2">
-        <f t="shared" ref="D65" si="161">C64-C65</f>
-        <v>192</v>
+        <f t="shared" ref="D65" si="163">C64-C65</f>
+        <v>200</v>
       </c>
       <c r="E65">
-        <f t="shared" ref="E65" si="162">$C$4-C65</f>
-        <v>5184</v>
+        <f t="shared" ref="E65" si="164">$C$4-C65</f>
+        <v>5192</v>
       </c>
       <c r="F65">
-        <f t="shared" ref="F65" si="163">$O$2-C65</f>
-        <v>-448</v>
+        <f t="shared" ref="F65" si="165">$O$2-C65</f>
+        <v>-440</v>
       </c>
       <c r="G65" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C66">
+        <v>33156</v>
+      </c>
+      <c r="D66" s="2">
+        <f t="shared" ref="D66" si="166">C65-C66</f>
+        <v>52</v>
+      </c>
+      <c r="E66">
+        <f t="shared" ref="E66" si="167">$C$4-C66</f>
+        <v>5244</v>
+      </c>
+      <c r="F66">
+        <f t="shared" ref="F66" si="168">$O$2-C66</f>
+        <v>-388</v>
+      </c>
+      <c r="G66" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C67">
+        <v>33092</v>
+      </c>
+      <c r="D67" s="2">
+        <f t="shared" ref="D67" si="169">C66-C67</f>
+        <v>64</v>
+      </c>
+      <c r="E67">
+        <f t="shared" ref="E67" si="170">$C$4-C67</f>
+        <v>5308</v>
+      </c>
+      <c r="F67">
+        <f t="shared" ref="F67" si="171">$O$2-C67</f>
+        <v>-324</v>
+      </c>
+      <c r="G67" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C68">
+        <v>32984</v>
+      </c>
+      <c r="D68" s="2">
+        <f t="shared" ref="D68" si="172">C67-C68</f>
+        <v>108</v>
+      </c>
+      <c r="E68">
+        <f t="shared" ref="E68" si="173">$C$4-C68</f>
+        <v>5416</v>
+      </c>
+      <c r="F68">
+        <f t="shared" ref="F68" si="174">$O$2-C68</f>
+        <v>-216</v>
+      </c>
+      <c r="G68" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C69">
+        <v>32996</v>
+      </c>
+      <c r="D69" s="2">
+        <f t="shared" ref="D69" si="175">C68-C69</f>
+        <v>-12</v>
+      </c>
+      <c r="E69">
+        <f t="shared" ref="E69" si="176">$C$4-C69</f>
+        <v>5404</v>
+      </c>
+      <c r="F69">
+        <f t="shared" ref="F69" si="177">$O$2-C69</f>
+        <v>-228</v>
+      </c>
+      <c r="G69" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
filtered white noise waveshapes gated by #ifdef, saving about 100 bytes.
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E862B35-6986-4B46-911A-7CE0907CFB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3BAE40-3305-4D59-846E-E1054CD81F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -247,6 +247,15 @@
   </si>
   <si>
     <t>de-inlining moog one pole filter</t>
+  </si>
+  <si>
+    <t>removing compensation gain on soft clipper which was also causing mbc problems</t>
+  </si>
+  <si>
+    <t>de-inline moog filter,'calculate filter G in function removing many clamps, misc</t>
+  </si>
+  <si>
+    <t>no filtered white noise wave  shapes.</t>
   </si>
 </sst>
 </file>
@@ -617,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2403,19 +2412,27 @@
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <f t="shared" ref="A66:A70" si="166">C66-$O$2</f>
+        <v>388</v>
+      </c>
+      <c r="B66" s="1" t="str">
+        <f t="shared" ref="B66:B70" si="167">REPT("#",A66*100/MAX(A:A))</f>
+        <v>######</v>
+      </c>
       <c r="C66">
         <v>33156</v>
       </c>
       <c r="D66" s="2">
-        <f t="shared" ref="D66" si="166">C65-C66</f>
+        <f t="shared" ref="D66" si="168">C65-C66</f>
         <v>52</v>
       </c>
       <c r="E66">
-        <f t="shared" ref="E66" si="167">$C$4-C66</f>
+        <f t="shared" ref="E66" si="169">$C$4-C66</f>
         <v>5244</v>
       </c>
       <c r="F66">
-        <f t="shared" ref="F66" si="168">$O$2-C66</f>
+        <f t="shared" ref="F66" si="170">$O$2-C66</f>
         <v>-388</v>
       </c>
       <c r="G66" t="s">
@@ -2423,19 +2440,27 @@
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <f t="shared" si="166"/>
+        <v>324</v>
+      </c>
+      <c r="B67" s="1" t="str">
+        <f t="shared" si="167"/>
+        <v>#####</v>
+      </c>
       <c r="C67">
         <v>33092</v>
       </c>
       <c r="D67" s="2">
-        <f t="shared" ref="D67" si="169">C66-C67</f>
+        <f t="shared" ref="D67" si="171">C66-C67</f>
         <v>64</v>
       </c>
       <c r="E67">
-        <f t="shared" ref="E67" si="170">$C$4-C67</f>
+        <f t="shared" ref="E67" si="172">$C$4-C67</f>
         <v>5308</v>
       </c>
       <c r="F67">
-        <f t="shared" ref="F67" si="171">$O$2-C67</f>
+        <f t="shared" ref="F67" si="173">$O$2-C67</f>
         <v>-324</v>
       </c>
       <c r="G67" t="s">
@@ -2443,19 +2468,27 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <f t="shared" si="166"/>
+        <v>216</v>
+      </c>
+      <c r="B68" s="1" t="str">
+        <f t="shared" si="167"/>
+        <v>###</v>
+      </c>
       <c r="C68">
         <v>32984</v>
       </c>
       <c r="D68" s="2">
-        <f t="shared" ref="D68" si="172">C67-C68</f>
+        <f t="shared" ref="D68" si="174">C67-C68</f>
         <v>108</v>
       </c>
       <c r="E68">
-        <f t="shared" ref="E68" si="173">$C$4-C68</f>
+        <f t="shared" ref="E68" si="175">$C$4-C68</f>
         <v>5416</v>
       </c>
       <c r="F68">
-        <f t="shared" ref="F68" si="174">$O$2-C68</f>
+        <f t="shared" ref="F68" si="176">$O$2-C68</f>
         <v>-216</v>
       </c>
       <c r="G68" t="s">
@@ -2463,23 +2496,99 @@
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <f t="shared" si="166"/>
+        <v>228</v>
+      </c>
+      <c r="B69" s="1" t="str">
+        <f t="shared" si="167"/>
+        <v>####</v>
+      </c>
       <c r="C69">
         <v>32996</v>
       </c>
       <c r="D69" s="2">
-        <f t="shared" ref="D69" si="175">C68-C69</f>
+        <f t="shared" ref="D69" si="177">C68-C69</f>
         <v>-12</v>
       </c>
       <c r="E69">
-        <f t="shared" ref="E69" si="176">$C$4-C69</f>
+        <f t="shared" ref="E69" si="178">$C$4-C69</f>
         <v>5404</v>
       </c>
       <c r="F69">
-        <f t="shared" ref="F69" si="177">$O$2-C69</f>
+        <f t="shared" ref="F69" si="179">$O$2-C69</f>
         <v>-228</v>
       </c>
       <c r="G69" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <f t="shared" si="166"/>
+        <v>212</v>
+      </c>
+      <c r="B70" s="1" t="str">
+        <f t="shared" si="167"/>
+        <v>###</v>
+      </c>
+      <c r="C70">
+        <v>32980</v>
+      </c>
+      <c r="D70" s="2">
+        <f t="shared" ref="D70" si="180">C69-C70</f>
+        <v>16</v>
+      </c>
+      <c r="E70">
+        <f t="shared" ref="E70" si="181">$C$4-C70</f>
+        <v>5420</v>
+      </c>
+      <c r="F70">
+        <f t="shared" ref="F70" si="182">$O$2-C70</f>
+        <v>-212</v>
+      </c>
+      <c r="G70" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C71">
+        <v>32960</v>
+      </c>
+      <c r="D71" s="2">
+        <f t="shared" ref="D71" si="183">C70-C71</f>
+        <v>20</v>
+      </c>
+      <c r="E71">
+        <f t="shared" ref="E71" si="184">$C$4-C71</f>
+        <v>5440</v>
+      </c>
+      <c r="F71">
+        <f t="shared" ref="F71" si="185">$O$2-C71</f>
+        <v>-192</v>
+      </c>
+      <c r="G71" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C72">
+        <v>32856</v>
+      </c>
+      <c r="D72" s="2">
+        <f t="shared" ref="D72" si="186">C71-C72</f>
+        <v>104</v>
+      </c>
+      <c r="E72">
+        <f t="shared" ref="E72" si="187">$C$4-C72</f>
+        <v>5544</v>
+      </c>
+      <c r="F72">
+        <f t="shared" ref="F72" si="188">$O$2-C72</f>
+        <v>-88</v>
+      </c>
+      <c r="G72" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WIP size optimizations: de-inlining things, moving calculations to param configs
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3BAE40-3305-4D59-846E-E1054CD81F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396B5767-8F58-44B2-B254-0D338FA85E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>no filtered white noise wave  shapes.</t>
+  </si>
+  <si>
+    <t>deinlining param stuff</t>
   </si>
 </sst>
 </file>
@@ -626,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O72"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2591,6 +2594,26 @@
         <v>76</v>
       </c>
     </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C73">
+        <v>32800</v>
+      </c>
+      <c r="D73" s="2">
+        <f t="shared" ref="D73" si="189">C72-C73</f>
+        <v>56</v>
+      </c>
+      <c r="E73">
+        <f t="shared" ref="E73" si="190">$C$4-C73</f>
+        <v>5600</v>
+      </c>
+      <c r="F73">
+        <f t="shared" ref="F73" si="191">$O$2-C73</f>
+        <v>-32</v>
+      </c>
+      <c r="G73" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
some more bytes saved
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396B5767-8F58-44B2-B254-0D338FA85E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{128B7A93-DF76-4FAE-9FF9-A99961BE2AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>deinlining param stuff</t>
+  </si>
+  <si>
+    <t>remove "square mode" from  sine wave shape, adding PM to fbm</t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O73"/>
+  <dimension ref="A1:O74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2555,19 +2558,27 @@
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <f t="shared" ref="A71:A73" si="183">C71-$O$2</f>
+        <v>192</v>
+      </c>
+      <c r="B71" s="1" t="str">
+        <f t="shared" ref="B71:B73" si="184">REPT("#",A71*100/MAX(A:A))</f>
+        <v>###</v>
+      </c>
       <c r="C71">
         <v>32960</v>
       </c>
       <c r="D71" s="2">
-        <f t="shared" ref="D71" si="183">C70-C71</f>
+        <f t="shared" ref="D71" si="185">C70-C71</f>
         <v>20</v>
       </c>
       <c r="E71">
-        <f t="shared" ref="E71" si="184">$C$4-C71</f>
+        <f t="shared" ref="E71" si="186">$C$4-C71</f>
         <v>5440</v>
       </c>
       <c r="F71">
-        <f t="shared" ref="F71" si="185">$O$2-C71</f>
+        <f t="shared" ref="F71" si="187">$O$2-C71</f>
         <v>-192</v>
       </c>
       <c r="G71" t="s">
@@ -2575,19 +2586,27 @@
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <f t="shared" si="183"/>
+        <v>88</v>
+      </c>
+      <c r="B72" s="1" t="str">
+        <f t="shared" si="184"/>
+        <v>#</v>
+      </c>
       <c r="C72">
         <v>32856</v>
       </c>
       <c r="D72" s="2">
-        <f t="shared" ref="D72" si="186">C71-C72</f>
+        <f t="shared" ref="D72" si="188">C71-C72</f>
         <v>104</v>
       </c>
       <c r="E72">
-        <f t="shared" ref="E72" si="187">$C$4-C72</f>
+        <f t="shared" ref="E72" si="189">$C$4-C72</f>
         <v>5544</v>
       </c>
       <c r="F72">
-        <f t="shared" ref="F72" si="188">$O$2-C72</f>
+        <f t="shared" ref="F72" si="190">$O$2-C72</f>
         <v>-88</v>
       </c>
       <c r="G72" t="s">
@@ -2595,23 +2614,51 @@
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <f t="shared" si="183"/>
+        <v>4</v>
+      </c>
+      <c r="B73" s="1" t="str">
+        <f t="shared" si="184"/>
+        <v/>
+      </c>
       <c r="C73">
-        <v>32800</v>
+        <v>32772</v>
       </c>
       <c r="D73" s="2">
-        <f t="shared" ref="D73" si="189">C72-C73</f>
-        <v>56</v>
+        <f t="shared" ref="D73" si="191">C72-C73</f>
+        <v>84</v>
       </c>
       <c r="E73">
-        <f t="shared" ref="E73" si="190">$C$4-C73</f>
-        <v>5600</v>
+        <f t="shared" ref="E73" si="192">$C$4-C73</f>
+        <v>5628</v>
       </c>
       <c r="F73">
-        <f t="shared" ref="F73" si="191">$O$2-C73</f>
-        <v>-32</v>
+        <f t="shared" ref="F73" si="193">$O$2-C73</f>
+        <v>-4</v>
       </c>
       <c r="G73" t="s">
         <v>77</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C74">
+        <v>32740</v>
+      </c>
+      <c r="D74" s="2">
+        <f t="shared" ref="D74" si="194">C73-C74</f>
+        <v>32</v>
+      </c>
+      <c r="E74">
+        <f t="shared" ref="E74" si="195">$C$4-C74</f>
+        <v>5660</v>
+      </c>
+      <c r="F74">
+        <f t="shared" ref="F74" si="196">$O$2-C74</f>
+        <v>28</v>
+      </c>
+      <c r="G74" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#149 voice stealing now properly resets voice states
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB1B6EB5-DBC6-467A-AE4F-9FFB5CDE94E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B098F0-16D8-4CBC-919E-3AA92A5D9C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -262,6 +262,9 @@
   </si>
   <si>
     <t>remove "square mode" from  sine wave shape, adding PM to fbm</t>
+  </si>
+  <si>
+    <t>fixing note stealing state</t>
   </si>
 </sst>
 </file>
@@ -632,13 +635,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O74"/>
+  <dimension ref="A1:O75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="6" customWidth="1"/>
+    <col min="5" max="5" width="6" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -663,13 +667,14 @@
         <v>5</v>
       </c>
       <c r="O2">
-        <v>32768</v>
+        <f>32768+140</f>
+        <v>32908</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A17" si="0">C3-$O$2</f>
-        <v>5120</v>
+        <v>4980</v>
       </c>
       <c r="B3" s="1" t="str">
         <f>REPT("#",A3*100/MAX(A:A))</f>
@@ -688,7 +693,7 @@
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>5632</v>
+        <v>5492</v>
       </c>
       <c r="B4" s="1" t="str">
         <f t="shared" ref="B4:B58" si="1">REPT("#",A4*100/MAX(A:A))</f>
@@ -703,7 +708,7 @@
       </c>
       <c r="F4">
         <f>$O$2-C4</f>
-        <v>-5632</v>
+        <v>-5492</v>
       </c>
       <c r="G4" t="s">
         <v>2</v>
@@ -712,7 +717,7 @@
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>5120</v>
+        <v>4980</v>
       </c>
       <c r="B5" s="1" t="str">
         <f t="shared" si="1"/>
@@ -731,7 +736,7 @@
       </c>
       <c r="F5">
         <f t="shared" ref="F5:F6" si="2">$O$2-C5</f>
-        <v>-5120</v>
+        <v>-4980</v>
       </c>
       <c r="G5" t="s">
         <v>3</v>
@@ -740,7 +745,7 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>4608</v>
+        <v>4468</v>
       </c>
       <c r="B6" s="1" t="str">
         <f t="shared" si="1"/>
@@ -759,7 +764,7 @@
       </c>
       <c r="F6">
         <f t="shared" si="2"/>
-        <v>-4608</v>
+        <v>-4468</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -768,11 +773,11 @@
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>4624</v>
+        <v>4484</v>
       </c>
       <c r="B7" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>##################################################################################</v>
+        <v>#################################################################################</v>
       </c>
       <c r="C7">
         <v>37392</v>
@@ -787,7 +792,7 @@
       </c>
       <c r="F7">
         <f>$O$2-C7</f>
-        <v>-4624</v>
+        <v>-4484</v>
       </c>
       <c r="G7" t="s">
         <v>10</v>
@@ -796,11 +801,11 @@
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>3868</v>
+        <v>3728</v>
       </c>
       <c r="B8" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>####################################################################</v>
+        <v>###################################################################</v>
       </c>
       <c r="C8">
         <v>36636</v>
@@ -815,7 +820,7 @@
       </c>
       <c r="F8">
         <f t="shared" ref="F8" si="5">$O$2-C8</f>
-        <v>-3868</v>
+        <v>-3728</v>
       </c>
       <c r="G8" t="s">
         <v>11</v>
@@ -824,11 +829,11 @@
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>3856</v>
+        <v>3716</v>
       </c>
       <c r="B9" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>####################################################################</v>
+        <v>###################################################################</v>
       </c>
       <c r="C9">
         <v>36624</v>
@@ -843,7 +848,7 @@
       </c>
       <c r="F9">
         <f t="shared" ref="F9" si="7">$O$2-C9</f>
-        <v>-3856</v>
+        <v>-3716</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
@@ -852,11 +857,11 @@
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>3864</v>
+        <v>3724</v>
       </c>
       <c r="B10" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>####################################################################</v>
+        <v>###################################################################</v>
       </c>
       <c r="C10">
         <v>36632</v>
@@ -871,7 +876,7 @@
       </c>
       <c r="F10">
         <f t="shared" ref="F10" si="9">$O$2-C10</f>
-        <v>-3864</v>
+        <v>-3724</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -880,7 +885,7 @@
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>3880</v>
+        <v>3740</v>
       </c>
       <c r="B11" s="1" t="str">
         <f t="shared" si="1"/>
@@ -899,7 +904,7 @@
       </c>
       <c r="F11">
         <f t="shared" ref="F11" si="11">$O$2-C11</f>
-        <v>-3880</v>
+        <v>-3740</v>
       </c>
       <c r="G11" t="s">
         <v>14</v>
@@ -908,11 +913,11 @@
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>3152</v>
+        <v>3012</v>
       </c>
       <c r="B12" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>#######################################################</v>
+        <v>######################################################</v>
       </c>
       <c r="C12">
         <v>35920</v>
@@ -927,7 +932,7 @@
       </c>
       <c r="F12">
         <f t="shared" ref="F12" si="13">$O$2-C12</f>
-        <v>-3152</v>
+        <v>-3012</v>
       </c>
       <c r="G12" t="s">
         <v>15</v>
@@ -936,11 +941,11 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>3076</v>
+        <v>2936</v>
       </c>
       <c r="B13" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>######################################################</v>
+        <v>#####################################################</v>
       </c>
       <c r="C13">
         <v>35844</v>
@@ -955,7 +960,7 @@
       </c>
       <c r="F13">
         <f t="shared" ref="F13" si="15">$O$2-C13</f>
-        <v>-3076</v>
+        <v>-2936</v>
       </c>
       <c r="G13" t="s">
         <v>16</v>
@@ -964,11 +969,11 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>3068</v>
+        <v>2928</v>
       </c>
       <c r="B14" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>######################################################</v>
+        <v>#####################################################</v>
       </c>
       <c r="C14">
         <v>35836</v>
@@ -983,7 +988,7 @@
       </c>
       <c r="F14">
         <f t="shared" ref="F14" si="17">$O$2-C14</f>
-        <v>-3068</v>
+        <v>-2928</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
@@ -992,11 +997,11 @@
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>2824</v>
+        <v>2684</v>
       </c>
       <c r="B15" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>##################################################</v>
+        <v>################################################</v>
       </c>
       <c r="C15">
         <v>35592</v>
@@ -1011,7 +1016,7 @@
       </c>
       <c r="F15">
         <f t="shared" ref="F15" si="19">$O$2-C15</f>
-        <v>-2824</v>
+        <v>-2684</v>
       </c>
       <c r="G15" t="s">
         <v>18</v>
@@ -1020,11 +1025,11 @@
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="0"/>
-        <v>1452</v>
+        <v>1312</v>
       </c>
       <c r="B16" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>#########################</v>
+        <v>#######################</v>
       </c>
       <c r="C16">
         <v>34220</v>
@@ -1039,7 +1044,7 @@
       </c>
       <c r="F16">
         <f t="shared" ref="F16" si="21">$O$2-C16</f>
-        <v>-1452</v>
+        <v>-1312</v>
       </c>
       <c r="G16" t="s">
         <v>19</v>
@@ -1048,11 +1053,11 @@
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="0"/>
-        <v>1512</v>
+        <v>1372</v>
       </c>
       <c r="B17" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>##########################</v>
+        <v>########################</v>
       </c>
       <c r="C17">
         <v>34280</v>
@@ -1067,7 +1072,7 @@
       </c>
       <c r="F17">
         <f t="shared" ref="F17" si="23">$O$2-C17</f>
-        <v>-1512</v>
+        <v>-1372</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1076,11 +1081,11 @@
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" ref="A18:A19" si="24">C18-$O$2</f>
-        <v>1508</v>
+        <v>1368</v>
       </c>
       <c r="B18" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>##########################</v>
+        <v>########################</v>
       </c>
       <c r="C18">
         <v>34276</v>
@@ -1095,7 +1100,7 @@
       </c>
       <c r="F18">
         <f t="shared" ref="F18" si="26">$O$2-C18</f>
-        <v>-1508</v>
+        <v>-1368</v>
       </c>
       <c r="G18" t="s">
         <v>21</v>
@@ -1104,11 +1109,11 @@
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="24"/>
-        <v>1424</v>
+        <v>1284</v>
       </c>
       <c r="B19" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>#########################</v>
+        <v>#######################</v>
       </c>
       <c r="C19">
         <v>34192</v>
@@ -1123,7 +1128,7 @@
       </c>
       <c r="F19">
         <f t="shared" ref="F19" si="28">$O$2-C19</f>
-        <v>-1424</v>
+        <v>-1284</v>
       </c>
       <c r="G19" t="s">
         <v>23</v>
@@ -1132,11 +1137,11 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" ref="A20:A21" si="29">C20-$O$2</f>
-        <v>1420</v>
+        <v>1280</v>
       </c>
       <c r="B20" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>#########################</v>
+        <v>#######################</v>
       </c>
       <c r="C20">
         <v>34188</v>
@@ -1151,7 +1156,7 @@
       </c>
       <c r="F20">
         <f t="shared" ref="F20" si="31">$O$2-C20</f>
-        <v>-1420</v>
+        <v>-1280</v>
       </c>
       <c r="G20" t="s">
         <v>24</v>
@@ -1160,11 +1165,11 @@
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="29"/>
-        <v>1364</v>
+        <v>1224</v>
       </c>
       <c r="B21" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>########################</v>
+        <v>######################</v>
       </c>
       <c r="C21">
         <v>34132</v>
@@ -1179,7 +1184,7 @@
       </c>
       <c r="F21">
         <f t="shared" ref="F21" si="33">$O$2-C21</f>
-        <v>-1364</v>
+        <v>-1224</v>
       </c>
       <c r="G21" t="s">
         <v>25</v>
@@ -1188,11 +1193,11 @@
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" ref="A22" si="34">C22-$O$2</f>
-        <v>1272</v>
+        <v>1132</v>
       </c>
       <c r="B22" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>######################</v>
+        <v>####################</v>
       </c>
       <c r="C22">
         <v>34040</v>
@@ -1207,7 +1212,7 @@
       </c>
       <c r="F22">
         <f t="shared" ref="F22" si="36">$O$2-C22</f>
-        <v>-1272</v>
+        <v>-1132</v>
       </c>
       <c r="G22" t="s">
         <v>26</v>
@@ -1216,11 +1221,11 @@
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" ref="A23" si="37">C23-$O$2</f>
-        <v>1256</v>
+        <v>1116</v>
       </c>
       <c r="B23" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>######################</v>
+        <v>####################</v>
       </c>
       <c r="C23">
         <v>34024</v>
@@ -1235,7 +1240,7 @@
       </c>
       <c r="F23">
         <f t="shared" ref="F23" si="39">$O$2-C23</f>
-        <v>-1256</v>
+        <v>-1116</v>
       </c>
       <c r="G23" t="s">
         <v>27</v>
@@ -1244,11 +1249,11 @@
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" ref="A24" si="40">C24-$O$2</f>
-        <v>1108</v>
+        <v>968</v>
       </c>
       <c r="B24" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>###################</v>
+        <v>#################</v>
       </c>
       <c r="C24">
         <v>33876</v>
@@ -1263,7 +1268,7 @@
       </c>
       <c r="F24">
         <f t="shared" ref="F24" si="42">$O$2-C24</f>
-        <v>-1108</v>
+        <v>-968</v>
       </c>
       <c r="G24" t="s">
         <v>28</v>
@@ -1272,7 +1277,7 @@
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" ref="A25:A26" si="43">C25-$O$2</f>
-        <v>-428</v>
+        <v>-568</v>
       </c>
       <c r="B25" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1291,7 +1296,7 @@
       </c>
       <c r="F25">
         <f t="shared" ref="F25" si="45">$O$2-C25</f>
-        <v>428</v>
+        <v>568</v>
       </c>
       <c r="G25" t="s">
         <v>29</v>
@@ -1300,7 +1305,7 @@
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="43"/>
-        <v>-132</v>
+        <v>-272</v>
       </c>
       <c r="B26" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1319,7 +1324,7 @@
       </c>
       <c r="F26">
         <f t="shared" ref="F26" si="47">$O$2-C26</f>
-        <v>132</v>
+        <v>272</v>
       </c>
       <c r="G26" t="s">
         <v>30</v>
@@ -1328,7 +1333,7 @@
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <f t="shared" ref="A27:A33" si="48">C27-$O$2</f>
-        <v>-56</v>
+        <v>-196</v>
       </c>
       <c r="B27" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1347,7 +1352,7 @@
       </c>
       <c r="F27">
         <f t="shared" ref="F27" si="50">$O$2-C27</f>
-        <v>56</v>
+        <v>196</v>
       </c>
       <c r="G27" t="s">
         <v>31</v>
@@ -1356,11 +1361,11 @@
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <f t="shared" si="48"/>
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="B28" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>##</v>
+        <v/>
       </c>
       <c r="C28">
         <v>32908</v>
@@ -1375,7 +1380,7 @@
       </c>
       <c r="F28">
         <f t="shared" ref="F28" si="52">$O$2-C28</f>
-        <v>-140</v>
+        <v>0</v>
       </c>
       <c r="G28" t="s">
         <v>32</v>
@@ -1384,11 +1389,11 @@
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <f t="shared" si="48"/>
-        <v>12</v>
-      </c>
-      <c r="B29" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-128</v>
+      </c>
+      <c r="B29" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C29">
         <v>32780</v>
@@ -1403,7 +1408,7 @@
       </c>
       <c r="F29">
         <f t="shared" ref="F29" si="54">$O$2-C29</f>
-        <v>-12</v>
+        <v>128</v>
       </c>
       <c r="G29" t="s">
         <v>33</v>
@@ -1412,7 +1417,7 @@
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <f t="shared" si="48"/>
-        <v>-32</v>
+        <v>-172</v>
       </c>
       <c r="B30" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1431,7 +1436,7 @@
       </c>
       <c r="F30">
         <f t="shared" ref="F30" si="56">$O$2-C30</f>
-        <v>32</v>
+        <v>172</v>
       </c>
       <c r="G30" t="s">
         <v>34</v>
@@ -1440,7 +1445,7 @@
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <f t="shared" si="48"/>
-        <v>-36</v>
+        <v>-176</v>
       </c>
       <c r="B31" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1459,7 +1464,7 @@
       </c>
       <c r="F31">
         <f t="shared" ref="F31" si="58">$O$2-C31</f>
-        <v>36</v>
+        <v>176</v>
       </c>
       <c r="G31" t="s">
         <v>35</v>
@@ -1468,11 +1473,11 @@
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <f t="shared" si="48"/>
-        <v>48</v>
-      </c>
-      <c r="B32" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-92</v>
+      </c>
+      <c r="B32" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C32">
         <v>32816</v>
@@ -1487,7 +1492,7 @@
       </c>
       <c r="F32">
         <f t="shared" ref="F32" si="60">$O$2-C32</f>
-        <v>-48</v>
+        <v>92</v>
       </c>
       <c r="G32" t="s">
         <v>36</v>
@@ -1496,11 +1501,11 @@
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <f t="shared" si="48"/>
-        <v>96</v>
-      </c>
-      <c r="B33" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>#</v>
+        <v>-44</v>
+      </c>
+      <c r="B33" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C33">
         <v>32864</v>
@@ -1515,7 +1520,7 @@
       </c>
       <c r="F33">
         <f t="shared" ref="F33" si="62">$O$2-C33</f>
-        <v>-96</v>
+        <v>44</v>
       </c>
       <c r="G33" t="s">
         <v>37</v>
@@ -1524,11 +1529,11 @@
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34">
         <f t="shared" ref="A34:A47" si="63">C34-$O$2</f>
-        <v>24</v>
-      </c>
-      <c r="B34" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-116</v>
+      </c>
+      <c r="B34" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C34">
         <v>32792</v>
@@ -1543,7 +1548,7 @@
       </c>
       <c r="F34">
         <f t="shared" ref="F34" si="65">$O$2-C34</f>
-        <v>-24</v>
+        <v>116</v>
       </c>
       <c r="G34" t="s">
         <v>38</v>
@@ -1552,11 +1557,11 @@
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
         <f t="shared" si="63"/>
-        <v>40</v>
-      </c>
-      <c r="B35" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-100</v>
+      </c>
+      <c r="B35" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C35">
         <v>32808</v>
@@ -1571,7 +1576,7 @@
       </c>
       <c r="F35">
         <f t="shared" ref="F35" si="68">$O$2-C35</f>
-        <v>-40</v>
+        <v>100</v>
       </c>
       <c r="G35" t="s">
         <v>39</v>
@@ -1580,11 +1585,11 @@
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <f t="shared" si="63"/>
-        <v>44</v>
-      </c>
-      <c r="B36" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-96</v>
+      </c>
+      <c r="B36" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C36">
         <v>32812</v>
@@ -1599,7 +1604,7 @@
       </c>
       <c r="F36">
         <f t="shared" ref="F36" si="71">$O$2-C36</f>
-        <v>-44</v>
+        <v>96</v>
       </c>
       <c r="G36" t="s">
         <v>40</v>
@@ -1608,11 +1613,11 @@
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <f t="shared" si="63"/>
-        <v>20</v>
-      </c>
-      <c r="B37" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-120</v>
+      </c>
+      <c r="B37" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C37">
         <v>32788</v>
@@ -1627,7 +1632,7 @@
       </c>
       <c r="F37">
         <f t="shared" ref="F37" si="74">$O$2-C37</f>
-        <v>-20</v>
+        <v>120</v>
       </c>
       <c r="G37" t="s">
         <v>41</v>
@@ -1636,11 +1641,11 @@
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <f t="shared" si="63"/>
-        <v>0</v>
-      </c>
-      <c r="B38" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-140</v>
+      </c>
+      <c r="B38" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C38">
         <v>32768</v>
@@ -1655,7 +1660,7 @@
       </c>
       <c r="F38">
         <f t="shared" ref="F38" si="77">$O$2-C38</f>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="G38" t="s">
         <v>42</v>
@@ -1664,7 +1669,7 @@
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <f t="shared" si="63"/>
-        <v>-56</v>
+        <v>-196</v>
       </c>
       <c r="B39" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1683,7 +1688,7 @@
       </c>
       <c r="F39">
         <f t="shared" ref="F39" si="80">$O$2-C39</f>
-        <v>56</v>
+        <v>196</v>
       </c>
       <c r="G39" t="s">
         <v>43</v>
@@ -1692,7 +1697,7 @@
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <f t="shared" si="63"/>
-        <v>-112</v>
+        <v>-252</v>
       </c>
       <c r="B40" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1711,7 +1716,7 @@
       </c>
       <c r="F40">
         <f t="shared" ref="F40" si="83">$O$2-C40</f>
-        <v>112</v>
+        <v>252</v>
       </c>
       <c r="G40" t="s">
         <v>44</v>
@@ -1720,7 +1725,7 @@
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <f t="shared" si="63"/>
-        <v>-96</v>
+        <v>-236</v>
       </c>
       <c r="B41" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1739,7 +1744,7 @@
       </c>
       <c r="F41">
         <f t="shared" ref="F41" si="86">$O$2-C41</f>
-        <v>96</v>
+        <v>236</v>
       </c>
       <c r="G41" t="s">
         <v>45</v>
@@ -1748,7 +1753,7 @@
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <f t="shared" si="63"/>
-        <v>-100</v>
+        <v>-240</v>
       </c>
       <c r="B42" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1767,7 +1772,7 @@
       </c>
       <c r="F42">
         <f t="shared" ref="F42" si="89">$O$2-C42</f>
-        <v>100</v>
+        <v>240</v>
       </c>
       <c r="G42" t="s">
         <v>46</v>
@@ -1776,7 +1781,7 @@
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <f t="shared" si="63"/>
-        <v>-80</v>
+        <v>-220</v>
       </c>
       <c r="B43" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1795,7 +1800,7 @@
       </c>
       <c r="F43">
         <f t="shared" ref="F43" si="92">$O$2-C43</f>
-        <v>80</v>
+        <v>220</v>
       </c>
       <c r="G43" t="s">
         <v>47</v>
@@ -1804,7 +1809,7 @@
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <f t="shared" si="63"/>
-        <v>-56</v>
+        <v>-196</v>
       </c>
       <c r="B44" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1823,7 +1828,7 @@
       </c>
       <c r="F44">
         <f t="shared" ref="F44" si="95">$O$2-C44</f>
-        <v>56</v>
+        <v>196</v>
       </c>
       <c r="G44" t="s">
         <v>48</v>
@@ -1832,11 +1837,11 @@
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
         <f t="shared" si="63"/>
-        <v>56</v>
-      </c>
-      <c r="B45" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-84</v>
+      </c>
+      <c r="B45" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C45">
         <v>32824</v>
@@ -1851,7 +1856,7 @@
       </c>
       <c r="F45">
         <f t="shared" ref="F45" si="98">$O$2-C45</f>
-        <v>-56</v>
+        <v>84</v>
       </c>
       <c r="G45" t="s">
         <v>49</v>
@@ -1860,7 +1865,7 @@
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
         <f t="shared" si="63"/>
-        <v>-12</v>
+        <v>-152</v>
       </c>
       <c r="B46" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1879,7 +1884,7 @@
       </c>
       <c r="F46">
         <f t="shared" ref="F46" si="101">$O$2-C46</f>
-        <v>12</v>
+        <v>152</v>
       </c>
       <c r="G46" t="s">
         <v>50</v>
@@ -1888,11 +1893,11 @@
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
         <f t="shared" si="63"/>
-        <v>36</v>
-      </c>
-      <c r="B47" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <v>-104</v>
+      </c>
+      <c r="B47" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C47">
         <v>32804</v>
@@ -1907,7 +1912,7 @@
       </c>
       <c r="F47">
         <f t="shared" ref="F47" si="104">$O$2-C47</f>
-        <v>-36</v>
+        <v>104</v>
       </c>
       <c r="G47" t="s">
         <v>51</v>
@@ -1916,7 +1921,7 @@
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
         <f t="shared" ref="A48:A54" si="105">C48-$O$2</f>
-        <v>-24</v>
+        <v>-164</v>
       </c>
       <c r="B48" s="1" t="e">
         <f t="shared" si="1"/>
@@ -1935,7 +1940,7 @@
       </c>
       <c r="F48">
         <f t="shared" ref="F48" si="108">$O$2-C48</f>
-        <v>24</v>
+        <v>164</v>
       </c>
       <c r="G48" t="s">
         <v>52</v>
@@ -1944,11 +1949,11 @@
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49">
         <f t="shared" si="105"/>
-        <v>344</v>
+        <v>204</v>
       </c>
       <c r="B49" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>######</v>
+        <v>###</v>
       </c>
       <c r="C49">
         <v>33112</v>
@@ -1963,7 +1968,7 @@
       </c>
       <c r="F49">
         <f t="shared" ref="F49" si="111">$O$2-C49</f>
-        <v>-344</v>
+        <v>-204</v>
       </c>
       <c r="G49" t="s">
         <v>53</v>
@@ -1972,11 +1977,11 @@
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50">
         <f t="shared" si="105"/>
-        <v>340</v>
+        <v>200</v>
       </c>
       <c r="B50" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>######</v>
+        <v>###</v>
       </c>
       <c r="C50">
         <v>33108</v>
@@ -1991,7 +1996,7 @@
       </c>
       <c r="F50">
         <f t="shared" ref="F50" si="114">$O$2-C50</f>
-        <v>-340</v>
+        <v>-200</v>
       </c>
       <c r="G50" t="s">
         <v>54</v>
@@ -2000,11 +2005,11 @@
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51">
         <f t="shared" si="105"/>
-        <v>296</v>
+        <v>156</v>
       </c>
       <c r="B51" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>#####</v>
+        <v>##</v>
       </c>
       <c r="C51">
         <v>33064</v>
@@ -2019,7 +2024,7 @@
       </c>
       <c r="F51">
         <f t="shared" ref="F51" si="117">$O$2-C51</f>
-        <v>-296</v>
+        <v>-156</v>
       </c>
       <c r="G51" t="s">
         <v>55</v>
@@ -2028,11 +2033,11 @@
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52">
         <f t="shared" si="105"/>
-        <v>256</v>
+        <v>116</v>
       </c>
       <c r="B52" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>####</v>
+        <v>##</v>
       </c>
       <c r="C52">
         <v>33024</v>
@@ -2047,7 +2052,7 @@
       </c>
       <c r="F52">
         <f t="shared" ref="F52" si="120">$O$2-C52</f>
-        <v>-256</v>
+        <v>-116</v>
       </c>
       <c r="G52" t="s">
         <v>56</v>
@@ -2056,11 +2061,11 @@
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53">
         <f t="shared" si="105"/>
-        <v>424</v>
+        <v>284</v>
       </c>
       <c r="B53" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>#######</v>
+        <v>#####</v>
       </c>
       <c r="C53">
         <v>33192</v>
@@ -2075,7 +2080,7 @@
       </c>
       <c r="F53">
         <f t="shared" ref="F53" si="123">$O$2-C53</f>
-        <v>-424</v>
+        <v>-284</v>
       </c>
       <c r="G53" t="s">
         <v>57</v>
@@ -2084,11 +2089,11 @@
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54">
         <f t="shared" si="105"/>
-        <v>256</v>
+        <v>116</v>
       </c>
       <c r="B54" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>####</v>
+        <v>##</v>
       </c>
       <c r="C54">
         <v>33024</v>
@@ -2103,7 +2108,7 @@
       </c>
       <c r="F54">
         <f t="shared" ref="F54" si="126">$O$2-C54</f>
-        <v>-256</v>
+        <v>-116</v>
       </c>
       <c r="G54" t="s">
         <v>58</v>
@@ -2112,11 +2117,11 @@
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55">
         <f t="shared" ref="A55:A56" si="127">C55-$O$2</f>
-        <v>232</v>
+        <v>92</v>
       </c>
       <c r="B55" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>####</v>
+        <v>#</v>
       </c>
       <c r="C55">
         <v>33000</v>
@@ -2131,7 +2136,7 @@
       </c>
       <c r="F55">
         <f t="shared" ref="F55" si="130">$O$2-C55</f>
-        <v>-232</v>
+        <v>-92</v>
       </c>
       <c r="G55" t="s">
         <v>59</v>
@@ -2140,11 +2145,11 @@
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56">
         <f t="shared" si="127"/>
-        <v>156</v>
+        <v>16</v>
       </c>
       <c r="B56" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>##</v>
+        <v/>
       </c>
       <c r="C56">
         <v>32924</v>
@@ -2159,7 +2164,7 @@
       </c>
       <c r="F56">
         <f t="shared" ref="F56" si="133">$O$2-C56</f>
-        <v>-156</v>
+        <v>-16</v>
       </c>
       <c r="G56" t="s">
         <v>60</v>
@@ -2168,11 +2173,11 @@
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57">
         <f t="shared" ref="A57:A58" si="134">C57-$O$2</f>
-        <v>132</v>
-      </c>
-      <c r="B57" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>##</v>
+        <v>-8</v>
+      </c>
+      <c r="B57" s="1" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
       </c>
       <c r="C57">
         <v>32900</v>
@@ -2187,7 +2192,7 @@
       </c>
       <c r="F57">
         <f t="shared" ref="F57" si="137">$O$2-C57</f>
-        <v>-132</v>
+        <v>8</v>
       </c>
       <c r="G57" t="s">
         <v>61</v>
@@ -2196,11 +2201,11 @@
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58">
         <f t="shared" si="134"/>
-        <v>196</v>
+        <v>56</v>
       </c>
       <c r="B58" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>###</v>
+        <v>#</v>
       </c>
       <c r="C58">
         <v>32964</v>
@@ -2215,7 +2220,7 @@
       </c>
       <c r="F58">
         <f t="shared" ref="F58" si="140">$O$2-C58</f>
-        <v>-196</v>
+        <v>-56</v>
       </c>
       <c r="G58" t="s">
         <v>62</v>
@@ -2224,11 +2229,11 @@
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59">
         <f t="shared" ref="A59:A60" si="141">C59-$O$2</f>
-        <v>152</v>
+        <v>12</v>
       </c>
       <c r="B59" s="1" t="str">
         <f t="shared" ref="B59:B60" si="142">REPT("#",A59*100/MAX(A:A))</f>
-        <v>##</v>
+        <v/>
       </c>
       <c r="C59">
         <v>32920</v>
@@ -2243,7 +2248,7 @@
       </c>
       <c r="F59">
         <f t="shared" ref="F59" si="145">$O$2-C59</f>
-        <v>-152</v>
+        <v>-12</v>
       </c>
       <c r="G59" t="s">
         <v>63</v>
@@ -2252,11 +2257,11 @@
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60">
         <f t="shared" si="141"/>
-        <v>72</v>
-      </c>
-      <c r="B60" s="1" t="str">
+        <v>-68</v>
+      </c>
+      <c r="B60" s="1" t="e">
         <f t="shared" si="142"/>
-        <v>#</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C60">
         <v>32840</v>
@@ -2271,7 +2276,7 @@
       </c>
       <c r="F60">
         <f t="shared" ref="F60" si="148">$O$2-C60</f>
-        <v>-72</v>
+        <v>68</v>
       </c>
       <c r="G60" t="s">
         <v>64</v>
@@ -2280,11 +2285,11 @@
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61">
         <f t="shared" ref="A61:A65" si="149">C61-$O$2</f>
-        <v>156</v>
+        <v>16</v>
       </c>
       <c r="B61" s="1" t="str">
         <f t="shared" ref="B61:B65" si="150">REPT("#",A61*100/MAX(A:A))</f>
-        <v>##</v>
+        <v/>
       </c>
       <c r="C61">
         <v>32924</v>
@@ -2299,7 +2304,7 @@
       </c>
       <c r="F61">
         <f t="shared" ref="F61" si="153">$O$2-C61</f>
-        <v>-156</v>
+        <v>-16</v>
       </c>
       <c r="G61" t="s">
         <v>65</v>
@@ -2308,11 +2313,11 @@
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62">
         <f t="shared" si="149"/>
-        <v>196</v>
+        <v>56</v>
       </c>
       <c r="B62" s="1" t="str">
         <f t="shared" si="150"/>
-        <v>###</v>
+        <v>#</v>
       </c>
       <c r="C62">
         <v>32964</v>
@@ -2327,7 +2332,7 @@
       </c>
       <c r="F62">
         <f t="shared" ref="F62" si="156">$O$2-C62</f>
-        <v>-196</v>
+        <v>-56</v>
       </c>
       <c r="G62" t="s">
         <v>66</v>
@@ -2336,11 +2341,11 @@
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63">
         <f t="shared" si="149"/>
-        <v>116</v>
-      </c>
-      <c r="B63" s="1" t="str">
+        <v>-24</v>
+      </c>
+      <c r="B63" s="1" t="e">
         <f t="shared" si="150"/>
-        <v>##</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C63">
         <v>32884</v>
@@ -2355,7 +2360,7 @@
       </c>
       <c r="F63">
         <f t="shared" ref="F63" si="159">$O$2-C63</f>
-        <v>-116</v>
+        <v>24</v>
       </c>
       <c r="G63" t="s">
         <v>67</v>
@@ -2364,11 +2369,11 @@
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64">
         <f t="shared" si="149"/>
-        <v>640</v>
+        <v>500</v>
       </c>
       <c r="B64" s="1" t="str">
         <f t="shared" si="150"/>
-        <v>###########</v>
+        <v>#########</v>
       </c>
       <c r="C64">
         <v>33408</v>
@@ -2383,7 +2388,7 @@
       </c>
       <c r="F64">
         <f t="shared" ref="F64" si="162">$O$2-C64</f>
-        <v>-640</v>
+        <v>-500</v>
       </c>
       <c r="G64" t="s">
         <v>68</v>
@@ -2392,11 +2397,11 @@
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65">
         <f t="shared" si="149"/>
-        <v>440</v>
+        <v>300</v>
       </c>
       <c r="B65" s="1" t="str">
         <f t="shared" si="150"/>
-        <v>#######</v>
+        <v>#####</v>
       </c>
       <c r="C65">
         <v>33208</v>
@@ -2411,7 +2416,7 @@
       </c>
       <c r="F65">
         <f t="shared" ref="F65" si="165">$O$2-C65</f>
-        <v>-440</v>
+        <v>-300</v>
       </c>
       <c r="G65" t="s">
         <v>69</v>
@@ -2420,11 +2425,11 @@
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
         <f t="shared" ref="A66:A70" si="166">C66-$O$2</f>
-        <v>388</v>
+        <v>248</v>
       </c>
       <c r="B66" s="1" t="str">
         <f t="shared" ref="B66:B70" si="167">REPT("#",A66*100/MAX(A:A))</f>
-        <v>######</v>
+        <v>####</v>
       </c>
       <c r="C66">
         <v>33156</v>
@@ -2439,7 +2444,7 @@
       </c>
       <c r="F66">
         <f t="shared" ref="F66" si="170">$O$2-C66</f>
-        <v>-388</v>
+        <v>-248</v>
       </c>
       <c r="G66" t="s">
         <v>70</v>
@@ -2448,11 +2453,11 @@
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67">
         <f t="shared" si="166"/>
-        <v>324</v>
+        <v>184</v>
       </c>
       <c r="B67" s="1" t="str">
         <f t="shared" si="167"/>
-        <v>#####</v>
+        <v>###</v>
       </c>
       <c r="C67">
         <v>33092</v>
@@ -2467,7 +2472,7 @@
       </c>
       <c r="F67">
         <f t="shared" ref="F67" si="173">$O$2-C67</f>
-        <v>-324</v>
+        <v>-184</v>
       </c>
       <c r="G67" t="s">
         <v>71</v>
@@ -2476,11 +2481,11 @@
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68">
         <f t="shared" si="166"/>
-        <v>216</v>
+        <v>76</v>
       </c>
       <c r="B68" s="1" t="str">
         <f t="shared" si="167"/>
-        <v>###</v>
+        <v>#</v>
       </c>
       <c r="C68">
         <v>32984</v>
@@ -2495,7 +2500,7 @@
       </c>
       <c r="F68">
         <f t="shared" ref="F68" si="176">$O$2-C68</f>
-        <v>-216</v>
+        <v>-76</v>
       </c>
       <c r="G68" t="s">
         <v>72</v>
@@ -2504,11 +2509,11 @@
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
         <f t="shared" si="166"/>
-        <v>228</v>
+        <v>88</v>
       </c>
       <c r="B69" s="1" t="str">
         <f t="shared" si="167"/>
-        <v>####</v>
+        <v>#</v>
       </c>
       <c r="C69">
         <v>32996</v>
@@ -2523,7 +2528,7 @@
       </c>
       <c r="F69">
         <f t="shared" ref="F69" si="179">$O$2-C69</f>
-        <v>-228</v>
+        <v>-88</v>
       </c>
       <c r="G69" t="s">
         <v>73</v>
@@ -2532,11 +2537,11 @@
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
         <f t="shared" si="166"/>
-        <v>212</v>
+        <v>72</v>
       </c>
       <c r="B70" s="1" t="str">
         <f t="shared" si="167"/>
-        <v>###</v>
+        <v>#</v>
       </c>
       <c r="C70">
         <v>32980</v>
@@ -2551,7 +2556,7 @@
       </c>
       <c r="F70">
         <f t="shared" ref="F70" si="182">$O$2-C70</f>
-        <v>-212</v>
+        <v>-72</v>
       </c>
       <c r="G70" t="s">
         <v>74</v>
@@ -2560,11 +2565,11 @@
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
         <f t="shared" ref="A71:A73" si="183">C71-$O$2</f>
-        <v>192</v>
+        <v>52</v>
       </c>
       <c r="B71" s="1" t="str">
         <f t="shared" ref="B71:B73" si="184">REPT("#",A71*100/MAX(A:A))</f>
-        <v>###</v>
+        <v/>
       </c>
       <c r="C71">
         <v>32960</v>
@@ -2579,7 +2584,7 @@
       </c>
       <c r="F71">
         <f t="shared" ref="F71" si="187">$O$2-C71</f>
-        <v>-192</v>
+        <v>-52</v>
       </c>
       <c r="G71" t="s">
         <v>75</v>
@@ -2588,11 +2593,11 @@
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
         <f t="shared" si="183"/>
-        <v>88</v>
-      </c>
-      <c r="B72" s="1" t="str">
+        <v>-52</v>
+      </c>
+      <c r="B72" s="1" t="e">
         <f t="shared" si="184"/>
-        <v>#</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C72">
         <v>32856</v>
@@ -2607,7 +2612,7 @@
       </c>
       <c r="F72">
         <f t="shared" ref="F72" si="190">$O$2-C72</f>
-        <v>-88</v>
+        <v>52</v>
       </c>
       <c r="G72" t="s">
         <v>76</v>
@@ -2616,11 +2621,11 @@
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
         <f t="shared" si="183"/>
-        <v>4</v>
-      </c>
-      <c r="B73" s="1" t="str">
+        <v>-136</v>
+      </c>
+      <c r="B73" s="1" t="e">
         <f t="shared" si="184"/>
-        <v/>
+        <v>#VALUE!</v>
       </c>
       <c r="C73">
         <v>32772</v>
@@ -2635,30 +2640,66 @@
       </c>
       <c r="F73">
         <f t="shared" ref="F73" si="193">$O$2-C73</f>
-        <v>-4</v>
+        <v>136</v>
       </c>
       <c r="G73" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <f t="shared" ref="A74:A75" si="194">C74-$O$2</f>
+        <v>-184</v>
+      </c>
+      <c r="B74" s="1" t="e">
+        <f t="shared" ref="B74:B75" si="195">REPT("#",A74*100/MAX(A:A))</f>
+        <v>#VALUE!</v>
+      </c>
       <c r="C74">
         <v>32724</v>
       </c>
       <c r="D74" s="2">
-        <f t="shared" ref="D74" si="194">C73-C74</f>
+        <f t="shared" ref="D74" si="196">C73-C74</f>
         <v>48</v>
       </c>
       <c r="E74">
-        <f t="shared" ref="E74" si="195">$C$4-C74</f>
+        <f t="shared" ref="E74" si="197">$C$4-C74</f>
         <v>5676</v>
       </c>
       <c r="F74">
-        <f t="shared" ref="F74" si="196">$O$2-C74</f>
-        <v>44</v>
+        <f t="shared" ref="F74" si="198">$O$2-C74</f>
+        <v>184</v>
       </c>
       <c r="G74" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <f t="shared" si="194"/>
+        <v>-32</v>
+      </c>
+      <c r="B75" s="1" t="e">
+        <f t="shared" si="195"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C75">
+        <v>32876</v>
+      </c>
+      <c r="D75" s="2">
+        <f t="shared" ref="D75" si="199">C74-C75</f>
+        <v>-152</v>
+      </c>
+      <c r="E75">
+        <f t="shared" ref="E75" si="200">$C$4-C75</f>
+        <v>5524</v>
+      </c>
+      <c r="F75">
+        <f t="shared" ref="F75" si="201">$O$2-C75</f>
+        <v>32</v>
+      </c>
+      <c r="G75" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixing imgui control ids for waveshape fixing mono never note-off
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B098F0-16D8-4CBC-919E-3AA92A5D9C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680433B8-08B1-4B9C-9465-3291FA5408A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>fixing note stealing state</t>
+  </si>
+  <si>
+    <t>#63 fixing more voice sync, fixing physically held prio</t>
   </si>
 </sst>
 </file>
@@ -635,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2702,6 +2705,34 @@
         <v>79</v>
       </c>
     </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <f t="shared" ref="A76" si="202">C76-$O$2</f>
+        <v>8</v>
+      </c>
+      <c r="B76" s="1" t="str">
+        <f t="shared" ref="B76" si="203">REPT("#",A76*100/MAX(A:A))</f>
+        <v/>
+      </c>
+      <c r="C76">
+        <v>32916</v>
+      </c>
+      <c r="D76" s="2">
+        <f t="shared" ref="D76" si="204">C75-C76</f>
+        <v>-40</v>
+      </c>
+      <c r="E76">
+        <f t="shared" ref="E76" si="205">$C$4-C76</f>
+        <v>5484</v>
+      </c>
+      <c r="F76">
+        <f t="shared" ref="F76" si="206">$O$2-C76</f>
+        <v>-8</v>
+      </c>
+      <c r="G76" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed broken oscillator filter state (#157)
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680433B8-08B1-4B9C-9465-3291FA5408A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5E0CF2-92E6-4061-A640-76B6DC00500E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -268,6 +268,18 @@
   </si>
   <si>
     <t>#63 fixing more voice sync, fixing physically held prio</t>
+  </si>
+  <si>
+    <t>opport:</t>
+  </si>
+  <si>
+    <t>butterw</t>
+  </si>
+  <si>
+    <t>width processing</t>
+  </si>
+  <si>
+    <t>fbm float precs?</t>
   </si>
 </sst>
 </file>
@@ -638,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O76"/>
+  <dimension ref="A1:O83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2733,6 +2745,26 @@
         <v>80</v>
       </c>
     </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G80" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="81" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G81" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="82" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G82" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="83" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G83" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
disabling pitchbend again fixing console exe: exit process, progress callback
</commit_message>
<xml_diff>
--- a/sizework20260301.xlsx
+++ b/sizework20260301.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\root\git\thenfour\WaveSabre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5E0CF2-92E6-4061-A640-76B6DC00500E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758E7BB7-1D89-4564-B262-ADE4FC39C03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11175" yWindow="1620" windowWidth="25005" windowHeight="16545" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{57C643F4-F52E-40AC-8074-51E8A42F966D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="85">
   <si>
     <t>with leveller, maj7space, mbc, maj7, 64-bit</t>
   </si>
@@ -270,16 +271,16 @@
     <t>#63 fixing more voice sync, fixing physically held prio</t>
   </si>
   <si>
-    <t>opport:</t>
-  </si>
-  <si>
-    <t>butterw</t>
-  </si>
-  <si>
-    <t>width processing</t>
-  </si>
-  <si>
-    <t>fbm float precs?</t>
+    <t>fixed osc resetting filter state, clamping filter hz, fixed voicing and legato, voice stealing, stereo width control</t>
+  </si>
+  <si>
+    <t>no imager</t>
+  </si>
+  <si>
+    <t>disable pitchbend</t>
+  </si>
+  <si>
+    <t>minor tweaks after testing console app (progress callback,…)</t>
   </si>
 </sst>
 </file>
@@ -650,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BF08B1-9BA5-43A8-9C7E-633386A766E4}">
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="74.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -2745,27 +2746,116 @@
         <v>80</v>
       </c>
     </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C77">
+        <v>33024</v>
+      </c>
+      <c r="D77" s="2">
+        <f t="shared" ref="D77" si="207">C76-C77</f>
+        <v>-108</v>
+      </c>
+      <c r="E77">
+        <f t="shared" ref="E77" si="208">$C$4-C77</f>
+        <v>5376</v>
+      </c>
+      <c r="F77">
+        <f t="shared" ref="F77" si="209">$O$2-C77</f>
+        <v>-116</v>
+      </c>
+      <c r="G77" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C78">
+        <v>32936</v>
+      </c>
+      <c r="D78" s="2">
+        <f t="shared" ref="D78" si="210">C77-C78</f>
+        <v>88</v>
+      </c>
+      <c r="E78">
+        <f t="shared" ref="E78" si="211">$C$4-C78</f>
+        <v>5464</v>
+      </c>
+      <c r="F78">
+        <f t="shared" ref="F78" si="212">$O$2-C78</f>
+        <v>-28</v>
+      </c>
+      <c r="G78" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C79">
+        <v>32708</v>
+      </c>
+      <c r="D79" s="2">
+        <f t="shared" ref="D79" si="213">C78-C79</f>
+        <v>228</v>
+      </c>
+      <c r="E79">
+        <f t="shared" ref="E79" si="214">$C$4-C79</f>
+        <v>5692</v>
+      </c>
+      <c r="F79">
+        <f t="shared" ref="F79" si="215">$O$2-C79</f>
+        <v>200</v>
+      </c>
+      <c r="G79" t="s">
+        <v>82</v>
+      </c>
+    </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C80">
+        <v>32708</v>
+      </c>
+      <c r="D80" s="2">
+        <f t="shared" ref="D80" si="216">C79-C80</f>
+        <v>0</v>
+      </c>
+      <c r="E80">
+        <f t="shared" ref="E80" si="217">$C$4-C80</f>
+        <v>5692</v>
+      </c>
+      <c r="F80">
+        <f t="shared" ref="F80" si="218">$O$2-C80</f>
+        <v>200</v>
+      </c>
       <c r="G80" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="81" spans="7:7" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="81" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C81">
+        <v>32760</v>
+      </c>
+      <c r="D81" s="2">
+        <f t="shared" ref="D81" si="219">C80-C81</f>
+        <v>-52</v>
+      </c>
+      <c r="E81">
+        <f t="shared" ref="E81" si="220">$C$4-C81</f>
+        <v>5640</v>
+      </c>
+      <c r="F81">
+        <f t="shared" ref="F81" si="221">$O$2-C81</f>
+        <v>148</v>
+      </c>
       <c r="G81" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="82" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G82" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="83" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G83" t="s">
         <v>84</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C42FA46-C395-40D3-849E-85E8997FBDEF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>